<commit_message>
chore: update RPS hash values [2026-05-28 19:57 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEF2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -99,6 +104,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2053,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2116,6 +2122,30 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-28 19:44:48</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-05-28 20:24 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2059,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2146,6 +2146,30 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-28 20:10:35</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-05-29 06:23 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2059,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2170,6 +2170,30 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-29 06:10:25</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-05-30 05:59 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2059,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2194,6 +2194,30 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-30 05:45:22</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-05-31 06:28 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2059,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2218,30 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-31 06:14:57</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 07:05 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2059,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2242,6 +2242,30 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01 06:52:01</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 11:19 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2059,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2266,6 +2266,30 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:05:20</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 11:41 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2059,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2290,6 +2290,30 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:28:34</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 11:58 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2059,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2314,6 +2314,30 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:45:11</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 12:40 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +68,11 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -95,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -105,6 +110,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -678,7 +684,11 @@
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
-      <c r="C24" s="3" t="n"/>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>a59d5c4f20b63854c4df3bed0310fbc2bee93af59c0a18d5e3a954e4d601fa20</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -696,7 +706,11 @@
         </is>
       </c>
       <c r="B26" s="2" t="n"/>
-      <c r="C26" s="3" t="n"/>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>8f5304ae2f1524f86cd781e21057001c1e3be04eda31d4469e88d0453e93c4b9</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -705,7 +719,11 @@
         </is>
       </c>
       <c r="B27" s="2" t="n"/>
-      <c r="C27" s="3" t="n"/>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>b49d363fea1698d0cbff18399767485ef9270ddbee1a1a7670e125462d0fab47</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -714,7 +732,11 @@
         </is>
       </c>
       <c r="B28" s="2" t="n"/>
-      <c r="C28" s="3" t="n"/>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -723,7 +745,11 @@
         </is>
       </c>
       <c r="B29" s="2" t="n"/>
-      <c r="C29" s="3" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>3648e39ea4020a4c625e5ab32c984527fa3a57fae67d0f069ca00c73e8cf2108</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -732,7 +758,11 @@
         </is>
       </c>
       <c r="B30" s="2" t="n"/>
-      <c r="C30" s="3" t="n"/>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>d8f3558dd1ac550c39aa10e9be6893687468f705c175768e30209db3c85a4c53</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -750,7 +780,11 @@
         </is>
       </c>
       <c r="B32" s="2" t="n"/>
-      <c r="C32" s="3" t="n"/>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>0c241186f021344adbd702a2597e4d322f38402077d02d4cb067154deca3c935</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -777,7 +811,11 @@
         </is>
       </c>
       <c r="B35" s="2" t="n"/>
-      <c r="C35" s="3" t="n"/>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>5d37089637de415d106d75fe99fe62d723ed7b89ef99a428890c802ab1c191b5</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -786,7 +824,11 @@
         </is>
       </c>
       <c r="B36" s="2" t="n"/>
-      <c r="C36" s="3" t="n"/>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>fc1c7d780c98b18ff17a0109a346316342ad815013763d1bd245c37b08b5c02b</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -849,7 +891,11 @@
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
-      <c r="C43" s="3" t="n"/>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>c1adf73082a14d642ad9d2f6151af5efab3d3d6531a018b71f3e5c60dfe8d75f</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -858,7 +904,11 @@
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
-      <c r="C44" s="3" t="n"/>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>5faecf12b7eb37185942d9c032d2327c8b32c5289aa0f7f0ef6e1b7090294289</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -867,7 +917,11 @@
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
-      <c r="C45" s="3" t="n"/>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>a14038d31708de4f8a5594ee7ca8166907baa31b2cd2e63811bb6fefb7b4c0a0</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -876,7 +930,11 @@
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
-      <c r="C46" s="3" t="n"/>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>f68f761f9f6c1ee104f780c7cf09c125c05aa1405a1f7d03a63e2ddf7d5820fc</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1074,7 +1132,11 @@
         </is>
       </c>
       <c r="B68" s="2" t="n"/>
-      <c r="C68" s="3" t="n"/>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>f8c54ae216a8851bcc87dcf7ddd411778580673fd1668726a6520e43591c5c93</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1119,7 +1181,11 @@
         </is>
       </c>
       <c r="B73" s="2" t="n"/>
-      <c r="C73" s="3" t="n"/>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>3ae9521463edeb0eced6c79ff99009318a605b4c1875f0764719306e04b1d6b6</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -1128,7 +1194,11 @@
         </is>
       </c>
       <c r="B74" s="2" t="n"/>
-      <c r="C74" s="3" t="n"/>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>7dae12401bb47769506966ad734f2330840383de6cb3853bd22cb145afcbe42c</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -1155,7 +1225,11 @@
         </is>
       </c>
       <c r="B77" s="2" t="n"/>
-      <c r="C77" s="3" t="n"/>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>d8f34f8159cd03ad5427029f244e099e16fc9360c9ac8ffa2c5dbead3b47159e</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -1164,7 +1238,11 @@
         </is>
       </c>
       <c r="B78" s="2" t="n"/>
-      <c r="C78" s="3" t="n"/>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>501f8dae7648ae91a810b9e2387294b2e8fe418312f99ff9b4f0f6caa7ffb7f2</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -1173,7 +1251,11 @@
         </is>
       </c>
       <c r="B79" s="2" t="n"/>
-      <c r="C79" s="3" t="n"/>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>fca0e583b4034a443821bda0f8672738cac6e91c078cc019c1969be960766078</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -1182,7 +1264,11 @@
         </is>
       </c>
       <c r="B80" s="2" t="n"/>
-      <c r="C80" s="3" t="n"/>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -1191,7 +1277,11 @@
         </is>
       </c>
       <c r="B81" s="2" t="n"/>
-      <c r="C81" s="3" t="n"/>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>78f4d0658968d9676c029dba90d3b95426f1e07ccf85a59586fabaad7c90e167</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -1200,7 +1290,11 @@
         </is>
       </c>
       <c r="B82" s="2" t="n"/>
-      <c r="C82" s="3" t="n"/>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>97abe1aac9218570b13169c1395f3ecd2651f8d2efa03e9b0c91b0da8f307afb</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -1209,7 +1303,11 @@
         </is>
       </c>
       <c r="B83" s="2" t="n"/>
-      <c r="C83" s="3" t="n"/>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>35c866a9bb3c47bb5d4f9332453c133e924f3932f83220aadeb413629f43ac62</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -1227,7 +1325,11 @@
         </is>
       </c>
       <c r="B85" s="2" t="n"/>
-      <c r="C85" s="3" t="n"/>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>3495c2faad0dc9d8a6f151c33ce11f7e60b1666b812ac20d8075e55e8e2ae20c</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -1245,7 +1347,11 @@
         </is>
       </c>
       <c r="B87" s="2" t="n"/>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>2d4327f484c5c1f2080dca40f9492c3fa6bfa0bb542764f35d2a84f55e1c27cd</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1254,7 +1360,11 @@
         </is>
       </c>
       <c r="B88" s="2" t="n"/>
-      <c r="C88" s="3" t="n"/>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>791423cc63028135230f287fa0af735437fd8ee36797c8f46e64e1cddd98e0ae</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -1263,7 +1373,11 @@
         </is>
       </c>
       <c r="B89" s="2" t="n"/>
-      <c r="C89" s="3" t="n"/>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -1272,7 +1386,11 @@
         </is>
       </c>
       <c r="B90" s="2" t="n"/>
-      <c r="C90" s="3" t="n"/>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -1290,7 +1408,11 @@
         </is>
       </c>
       <c r="B92" s="2" t="n"/>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1317,7 +1439,11 @@
         </is>
       </c>
       <c r="B95" s="2" t="n"/>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1326,7 +1452,11 @@
         </is>
       </c>
       <c r="B96" s="2" t="n"/>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1335,7 +1465,11 @@
         </is>
       </c>
       <c r="B97" s="2" t="n"/>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1353,7 +1487,11 @@
         </is>
       </c>
       <c r="B99" s="2" t="n"/>
-      <c r="C99" s="3" t="n"/>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>51b08ef9938bb45ef673804ba89c5e5eea02391599e8736362ae7626dff1ed94</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -1362,7 +1500,11 @@
         </is>
       </c>
       <c r="B100" s="2" t="n"/>
-      <c r="C100" s="3" t="n"/>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>be6ec70b8a7f46f7d6a06b554ecf50a16d437e6fcc62de6201fc88ef77c8e589</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -1380,7 +1522,11 @@
         </is>
       </c>
       <c r="B102" s="2" t="n"/>
-      <c r="C102" s="3" t="n"/>
+      <c r="C102" s="7" t="inlineStr">
+        <is>
+          <t>8305796017bbaf420b6513131705df553987508840f6d6d3a9c273856bce6a88</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -1389,7 +1535,11 @@
         </is>
       </c>
       <c r="B103" s="2" t="n"/>
-      <c r="C103" s="3" t="n"/>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>d518580384830d59c4970219d50dba21d7f0b9f198158f96e429430b3da34738</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -1398,7 +1548,11 @@
         </is>
       </c>
       <c r="B104" s="2" t="n"/>
-      <c r="C104" s="3" t="n"/>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>81f0db78033949cad3ca3573547710a1b699b59edb88b8bc054053f87032684e</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -1407,7 +1561,11 @@
         </is>
       </c>
       <c r="B105" s="2" t="n"/>
-      <c r="C105" s="3" t="n"/>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -1434,7 +1592,11 @@
         </is>
       </c>
       <c r="B108" s="2" t="n"/>
-      <c r="C108" s="3" t="n"/>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>f95600dbe4b7515fad7acde4481cc0cce4decf85732e935968f8d2b0f9d293a1</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -1452,7 +1614,11 @@
         </is>
       </c>
       <c r="B110" s="2" t="n"/>
-      <c r="C110" s="3" t="n"/>
+      <c r="C110" s="7" t="inlineStr">
+        <is>
+          <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -1461,7 +1627,11 @@
         </is>
       </c>
       <c r="B111" s="2" t="n"/>
-      <c r="C111" s="3" t="n"/>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>66e1bef0bd7b07e2497af494d0c4a293672323135f876763fdf12792132d8a22</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -1470,7 +1640,11 @@
         </is>
       </c>
       <c r="B112" s="2" t="n"/>
-      <c r="C112" s="3" t="n"/>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>b4471a9a0184a21afb00ed648b5850b0828fc314f5b4cae05a5baf17dd62ce06</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -1488,7 +1662,11 @@
         </is>
       </c>
       <c r="B114" s="2" t="n"/>
-      <c r="C114" s="3" t="n"/>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>db305a14a585151ef7c215b3f9b378664b2eb4b3e871056308243818a6038dc4</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -1497,7 +1675,11 @@
         </is>
       </c>
       <c r="B115" s="2" t="n"/>
-      <c r="C115" s="3" t="n"/>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>dbeac7ceb2efa6046986b3277977fbedd6a46b087b148a31c3917fa47acc50a3</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -1506,7 +1688,11 @@
         </is>
       </c>
       <c r="B116" s="2" t="n"/>
-      <c r="C116" s="3" t="n"/>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>6534abc9a6ec370e98171e10302ac7098e92763d88fc2b73859a865ec21b352a</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -1515,7 +1701,11 @@
         </is>
       </c>
       <c r="B117" s="2" t="n"/>
-      <c r="C117" s="3" t="n"/>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>f2a539248a18f0e2c14ce9bf1844814b3d299d0437b34c5bc9389552d7cf921b</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -1542,7 +1732,11 @@
         </is>
       </c>
       <c r="B120" s="2" t="n"/>
-      <c r="C120" s="3" t="n"/>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>c77698286bc91feca5d67a11f6d92f9e4aa427bf32b5b18bf7c4cb91b5ede995</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -1551,7 +1745,11 @@
         </is>
       </c>
       <c r="B121" s="2" t="n"/>
-      <c r="C121" s="3" t="n"/>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -1569,7 +1767,11 @@
         </is>
       </c>
       <c r="B123" s="2" t="n"/>
-      <c r="C123" s="3" t="n"/>
+      <c r="C123" s="7" t="inlineStr">
+        <is>
+          <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -1587,7 +1789,11 @@
         </is>
       </c>
       <c r="B125" s="2" t="n"/>
-      <c r="C125" s="3" t="n"/>
+      <c r="C125" s="7" t="inlineStr">
+        <is>
+          <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -1614,7 +1820,11 @@
         </is>
       </c>
       <c r="B128" s="2" t="n"/>
-      <c r="C128" s="3" t="n"/>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>123eff993c9338db4825258e12a99915dd30c2dfaa85d2bd722eb4aa7fa934a8</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -1641,7 +1851,11 @@
         </is>
       </c>
       <c r="B131" s="2" t="n"/>
-      <c r="C131" s="3" t="n"/>
+      <c r="C131" s="7" t="inlineStr">
+        <is>
+          <t>c339d5a4c816c8fe640bb33245ee683bbe1a03ddecbd211cd33b5770b2ff3bee</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -1650,7 +1864,11 @@
         </is>
       </c>
       <c r="B132" s="2" t="n"/>
-      <c r="C132" s="3" t="n"/>
+      <c r="C132" s="7" t="inlineStr">
+        <is>
+          <t>6ad1c795d9459f2cfe15aac0c268ada6ca5eb2af707b379d525f43f76baaeecd</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -1659,7 +1877,11 @@
         </is>
       </c>
       <c r="B133" s="2" t="n"/>
-      <c r="C133" s="3" t="n"/>
+      <c r="C133" s="7" t="inlineStr">
+        <is>
+          <t>286743119741e3d8569d95f3a661d97f580208f5dcdfe028c3fb0dc9c73fd511</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -1668,7 +1890,11 @@
         </is>
       </c>
       <c r="B134" s="2" t="n"/>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
+          <t>3dcb502f532343574ae604f9293110487e36dcb657946afe8b6cf4b8d2676ec3</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -1677,7 +1903,11 @@
         </is>
       </c>
       <c r="B135" s="2" t="n"/>
-      <c r="C135" s="3" t="n"/>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t>5e4a8fa56aad55b9202fcc9a27f2cdcc4c633fee759c57cc555eb8c37672d8aa</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -1704,7 +1934,11 @@
         </is>
       </c>
       <c r="B138" s="2" t="n"/>
-      <c r="C138" s="3" t="n"/>
+      <c r="C138" s="7" t="inlineStr">
+        <is>
+          <t>661b722535b10cdf0de28fa5864d8c1c864c1c6f60b7b6c8e98e793ad73aff4e</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -1731,7 +1965,11 @@
         </is>
       </c>
       <c r="B141" s="2" t="n"/>
-      <c r="C141" s="3" t="n"/>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t>c32fc899559630a399ab8c58c81bcd18273925656dfeba91aa0b780795c122de</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -1740,7 +1978,11 @@
         </is>
       </c>
       <c r="B142" s="2" t="n"/>
-      <c r="C142" s="3" t="n"/>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t>1868912449868cc8572bc8ff350dda7706018bb79c95ed9bd84b486e3ff293eb</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -1803,7 +2045,11 @@
         </is>
       </c>
       <c r="B149" s="2" t="n"/>
-      <c r="C149" s="3" t="n"/>
+      <c r="C149" s="7" t="inlineStr">
+        <is>
+          <t>25b89a575dc4068f1dfec36d7ba1a3d5fe2494aff373a8a56da95394b68e5665</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -1812,7 +2058,11 @@
         </is>
       </c>
       <c r="B150" s="2" t="n"/>
-      <c r="C150" s="3" t="n"/>
+      <c r="C150" s="7" t="inlineStr">
+        <is>
+          <t>93e0500aba96ec8070238428036e3b086ba000b945defae61b5c4bb9f82f6fe2</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -1839,7 +2089,11 @@
         </is>
       </c>
       <c r="B153" s="2" t="n"/>
-      <c r="C153" s="3" t="n"/>
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -1848,7 +2102,11 @@
         </is>
       </c>
       <c r="B154" s="2" t="n"/>
-      <c r="C154" s="3" t="n"/>
+      <c r="C154" s="7" t="inlineStr">
+        <is>
+          <t>0c2763e4cbb15e86537a56cc3876313f65777ca39f265ec814950470fb611097</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -1857,7 +2115,11 @@
         </is>
       </c>
       <c r="B155" s="2" t="n"/>
-      <c r="C155" s="3" t="n"/>
+      <c r="C155" s="7" t="inlineStr">
+        <is>
+          <t>b1ceda46805367b39634e4c4c7cc43c3220072f4f0ecaf8d1d32c2541725ad05</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -1884,7 +2146,11 @@
         </is>
       </c>
       <c r="B158" s="2" t="n"/>
-      <c r="C158" s="3" t="n"/>
+      <c r="C158" s="7" t="inlineStr">
+        <is>
+          <t>26da235ced9cc83f9bb8e10c17e32985abea89a92308573ce687e82f3f04a8ee</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -1974,7 +2240,11 @@
         </is>
       </c>
       <c r="B168" s="2" t="n"/>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="7" t="inlineStr">
+        <is>
+          <t>2748bfdae093fc22c38d7699d0eff0027b36ddf5e474388d9ea5a6e350a445e1</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -1983,7 +2253,11 @@
         </is>
       </c>
       <c r="B169" s="2" t="n"/>
-      <c r="C169" s="3" t="n"/>
+      <c r="C169" s="7" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -1992,7 +2266,11 @@
         </is>
       </c>
       <c r="B170" s="2" t="n"/>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="7" t="inlineStr">
+        <is>
+          <t>00c79ba93df9be776984c966c36f797929bd6a347c893f65a4ef8567333a9741</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2019,7 +2297,11 @@
         </is>
       </c>
       <c r="B173" s="2" t="n"/>
-      <c r="C173" s="3" t="n"/>
+      <c r="C173" s="7" t="inlineStr">
+        <is>
+          <t>20b6f000a58e180c0b81853a00e148d6b13055577deebdf160357c20623f1856</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -2028,7 +2310,11 @@
         </is>
       </c>
       <c r="B174" s="2" t="n"/>
-      <c r="C174" s="3" t="n"/>
+      <c r="C174" s="7" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -2059,7 +2345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2338,6 +2624,30 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:27:23</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 13:11 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +73,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -100,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -111,6 +116,8 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,10 +690,14 @@
           <t>DOS_SDP</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>a59d5c4f20b63854c4df3bed0310fbc2bee93af59c0a18d5e3a954e4d601fa20</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>e8809bef06e7b2733e46f1d7ab56c848be1d7dbd6d7af0808004ffca15481f31</t>
         </is>
       </c>
     </row>
@@ -705,10 +716,14 @@
           <t>EE_FSA_IA</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>8f5304ae2f1524f86cd781e21057001c1e3be04eda31d4469e88d0453e93c4b9</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
         </is>
       </c>
     </row>
@@ -718,10 +733,14 @@
           <t>EE_MFA_BELARUS</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>b49d363fea1698d0cbff18399767485ef9270ddbee1a1a7670e125462d0fab47</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>8f5304ae2f1524f86cd781e21057001c1e3be04eda31d4469e88d0453e93c4b9</t>
         </is>
       </c>
     </row>
@@ -731,10 +750,14 @@
           <t>EE_MFA_HR</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>d8f3558dd1ac550c39aa10e9be6893687468f705c175768e30209db3c85a4c53</t>
         </is>
       </c>
     </row>
@@ -744,10 +767,14 @@
           <t>EE_MFA_RUSSIA</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>3648e39ea4020a4c625e5ab32c984527fa3a57fae67d0f069ca00c73e8cf2108</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>af0ba49273abf20fc9ad6a958c30545abe715f6dc086c82b8f42f8ffc293693a</t>
         </is>
       </c>
     </row>
@@ -757,10 +784,14 @@
           <t>ES_BOS_SANCTIONS</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>d8f3558dd1ac550c39aa10e9be6893687468f705c175768e30209db3c85a4c53</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>e89f3f0ef4c85b90f58f5699acd19a0b412df4204c446142abe65d3e72d8792e</t>
         </is>
       </c>
     </row>
@@ -779,12 +810,12 @@
           <t>ES_WA_CNMV</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>0c241186f021344adbd702a2597e4d322f38402077d02d4cb067154deca3c935</t>
         </is>
       </c>
+      <c r="C32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -810,10 +841,14 @@
           <t>EU_ECB_SANCTIONS</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>5d37089637de415d106d75fe99fe62d723ed7b89ef99a428890c802ab1c191b5</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>e4fd0143e2c774595c60b307396849dcd3b6d001cc3dbdc82ba7c3557f9aa3e0</t>
         </is>
       </c>
     </row>
@@ -823,8 +858,12 @@
           <t>EU_EIB_LOE</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>fc1c7d780c98b18ff17a0109a346316342ad815013763d1bd245c37b08b5c02b</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>fc1c7d780c98b18ff17a0109a346316342ad815013763d1bd245c37b08b5c02b</t>
         </is>
@@ -890,10 +929,14 @@
           <t>GB_OFSI_TR_MP</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>c1adf73082a14d642ad9d2f6151af5efab3d3d6531a018b71f3e5c60dfe8d75f</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>727002db8d4a852527360740f82788109fe7990d5fa865436f209de32dcc55e7</t>
         </is>
       </c>
     </row>
@@ -903,10 +946,14 @@
           <t>GE_MOJ_OTKHOZORIA_TATUNASHVILI_LIST</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>5faecf12b7eb37185942d9c032d2327c8b32c5289aa0f7f0ef6e1b7090294289</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>9ae7d6ec85e9dc4953355a9e61bd3d799eac5b91115e1e13c8383d17e25046b1</t>
         </is>
       </c>
     </row>
@@ -916,10 +963,14 @@
           <t>GG_GFSC_DD</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>a14038d31708de4f8a5594ee7ca8166907baa31b2cd2e63811bb6fefb7b4c0a0</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>4aa0007d8931b3893d0f7c946b8120fa5ea848590744cabd2fde3467a5fbc7e1</t>
         </is>
       </c>
     </row>
@@ -929,10 +980,14 @@
           <t>HK_ICAC_WL</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>f68f761f9f6c1ee104f780c7cf09c125c05aa1405a1f7d03a63e2ddf7d5820fc</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>c1adf73082a14d642ad9d2f6151af5efab3d3d6531a018b71f3e5c60dfe8d75f</t>
         </is>
       </c>
     </row>
@@ -961,7 +1016,11 @@
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
-      <c r="C49" s="3" t="n"/>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>334adc9bfc7a3169bfb68adab22e292eabb343df6b26689e0a83eb626575f0f4</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1131,12 +1190,12 @@
           <t>KE_FRC_DTFS</t>
         </is>
       </c>
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="7" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>f8c54ae216a8851bcc87dcf7ddd411778580673fd1668726a6520e43591c5c93</t>
         </is>
       </c>
+      <c r="C68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1172,7 +1231,11 @@
         </is>
       </c>
       <c r="B72" s="2" t="n"/>
-      <c r="C72" s="3" t="n"/>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>e9dcf5df0a9cdafc102ba5cd0bc59d21fd8f4f306cc23a906e3f5d0e6d94ae5e</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -1180,10 +1243,14 @@
           <t>LV_FIU_SANCTIONED_SUBJECTS</t>
         </is>
       </c>
-      <c r="B73" s="2" t="n"/>
-      <c r="C73" s="7" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>3ae9521463edeb0eced6c79ff99009318a605b4c1875f0764719306e04b1d6b6</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>7dae12401bb47769506966ad734f2330840383de6cb3853bd22cb145afcbe42c</t>
         </is>
       </c>
     </row>
@@ -1193,12 +1260,12 @@
           <t>MC_BT_NAFL</t>
         </is>
       </c>
-      <c r="B74" s="2" t="n"/>
-      <c r="C74" s="7" t="inlineStr">
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>7dae12401bb47769506966ad734f2330840383de6cb3853bd22cb145afcbe42c</t>
         </is>
       </c>
+      <c r="C74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -1224,10 +1291,14 @@
           <t>MY_BNM_WANTED</t>
         </is>
       </c>
-      <c r="B77" s="2" t="n"/>
-      <c r="C77" s="7" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>d8f34f8159cd03ad5427029f244e099e16fc9360c9ac8ffa2c5dbead3b47159e</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>501f8dae7648ae91a810b9e2387294b2e8fe418312f99ff9b4f0f6caa7ffb7f2</t>
         </is>
       </c>
     </row>
@@ -1237,10 +1308,14 @@
           <t>MY_BNM_WARNING_LETTERS</t>
         </is>
       </c>
-      <c r="B78" s="2" t="n"/>
-      <c r="C78" s="7" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>501f8dae7648ae91a810b9e2387294b2e8fe418312f99ff9b4f0f6caa7ffb7f2</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>78f4d0658968d9676c029dba90d3b95426f1e07ccf85a59586fabaad7c90e167</t>
         </is>
       </c>
     </row>
@@ -1250,10 +1325,14 @@
           <t>MY_MHA_MOHA_LIST</t>
         </is>
       </c>
-      <c r="B79" s="2" t="n"/>
-      <c r="C79" s="7" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>fca0e583b4034a443821bda0f8672738cac6e91c078cc019c1969be960766078</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>d8f34f8159cd03ad5427029f244e099e16fc9360c9ac8ffa2c5dbead3b47159e</t>
         </is>
       </c>
     </row>
@@ -1263,8 +1342,12 @@
           <t>MY_SCM_IA</t>
         </is>
       </c>
-      <c r="B80" s="2" t="n"/>
-      <c r="C80" s="7" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
         <is>
           <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
         </is>
@@ -1276,10 +1359,14 @@
           <t>MY_SCM_WANTED</t>
         </is>
       </c>
-      <c r="B81" s="2" t="n"/>
-      <c r="C81" s="7" t="inlineStr">
+      <c r="B81" s="2" t="inlineStr">
         <is>
           <t>78f4d0658968d9676c029dba90d3b95426f1e07ccf85a59586fabaad7c90e167</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>fca0e583b4034a443821bda0f8672738cac6e91c078cc019c1969be960766078</t>
         </is>
       </c>
     </row>
@@ -1289,8 +1376,12 @@
           <t>NG_EFCC_WANTED_PERSON</t>
         </is>
       </c>
-      <c r="B82" s="2" t="n"/>
-      <c r="C82" s="7" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>97abe1aac9218570b13169c1395f3ecd2651f8d2efa03e9b0c91b0da8f307afb</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
         <is>
           <t>97abe1aac9218570b13169c1395f3ecd2651f8d2efa03e9b0c91b0da8f307afb</t>
         </is>
@@ -1302,8 +1393,12 @@
           <t>NG_NIGSAC_ENTITIES</t>
         </is>
       </c>
-      <c r="B83" s="2" t="n"/>
-      <c r="C83" s="7" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>35c866a9bb3c47bb5d4f9332453c133e924f3932f83220aadeb413629f43ac62</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
         <is>
           <t>35c866a9bb3c47bb5d4f9332453c133e924f3932f83220aadeb413629f43ac62</t>
         </is>
@@ -1324,8 +1419,12 @@
           <t>NO_BLACK_LIST</t>
         </is>
       </c>
-      <c r="B85" s="2" t="n"/>
-      <c r="C85" s="7" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>3495c2faad0dc9d8a6f151c33ce11f7e60b1666b812ac20d8075e55e8e2ae20c</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
         <is>
           <t>3495c2faad0dc9d8a6f151c33ce11f7e60b1666b812ac20d8075e55e8e2ae20c</t>
         </is>
@@ -1346,10 +1445,14 @@
           <t>OIG_MOST_WANTED</t>
         </is>
       </c>
-      <c r="B87" s="2" t="n"/>
-      <c r="C87" s="7" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>2d4327f484c5c1f2080dca40f9492c3fa6bfa0bb542764f35d2a84f55e1c27cd</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>791423cc63028135230f287fa0af735437fd8ee36797c8f46e64e1cddd98e0ae</t>
         </is>
       </c>
     </row>
@@ -1359,10 +1462,14 @@
           <t>OM_NCTC_LL</t>
         </is>
       </c>
-      <c r="B88" s="2" t="n"/>
-      <c r="C88" s="7" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>791423cc63028135230f287fa0af735437fd8ee36797c8f46e64e1cddd98e0ae</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
     </row>
@@ -1372,10 +1479,14 @@
           <t>PA_TREAS_SCI</t>
         </is>
       </c>
-      <c r="B89" s="2" t="n"/>
-      <c r="C89" s="7" t="inlineStr">
+      <c r="B89" s="2" t="inlineStr">
         <is>
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>2d4327f484c5c1f2080dca40f9492c3fa6bfa0bb542764f35d2a84f55e1c27cd</t>
         </is>
       </c>
     </row>
@@ -1385,12 +1496,12 @@
           <t>PE_MEF_DISQUALIFIED_SUPPLIERS</t>
         </is>
       </c>
-      <c r="B90" s="2" t="n"/>
-      <c r="C90" s="7" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
         </is>
       </c>
+      <c r="C90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -1399,7 +1510,11 @@
         </is>
       </c>
       <c r="B91" s="2" t="n"/>
-      <c r="C91" s="3" t="n"/>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -1407,10 +1522,14 @@
           <t>PRM_AK_DHSS_EPL</t>
         </is>
       </c>
-      <c r="B92" s="2" t="n"/>
-      <c r="C92" s="7" t="inlineStr">
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>51b08ef9938bb45ef673804ba89c5e5eea02391599e8736362ae7626dff1ed94</t>
         </is>
       </c>
     </row>
@@ -1438,10 +1557,14 @@
           <t>PRM_CA_DHCS_SIPL</t>
         </is>
       </c>
-      <c r="B95" s="2" t="n"/>
-      <c r="C95" s="7" t="inlineStr">
+      <c r="B95" s="2" t="inlineStr">
         <is>
           <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
         </is>
       </c>
     </row>
@@ -1451,8 +1574,12 @@
           <t>PRM_CA_DIR_DC</t>
         </is>
       </c>
-      <c r="B96" s="2" t="n"/>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="inlineStr">
         <is>
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
@@ -1464,8 +1591,12 @@
           <t>PRM_DC_DDS_PSL</t>
         </is>
       </c>
-      <c r="B97" s="2" t="n"/>
-      <c r="C97" s="7" t="inlineStr">
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
         <is>
           <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
         </is>
@@ -1486,10 +1617,14 @@
           <t>PRM_GA_DCH_EIE</t>
         </is>
       </c>
-      <c r="B99" s="2" t="n"/>
-      <c r="C99" s="7" t="inlineStr">
+      <c r="B99" s="2" t="inlineStr">
         <is>
           <t>51b08ef9938bb45ef673804ba89c5e5eea02391599e8736362ae7626dff1ed94</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
         </is>
       </c>
     </row>
@@ -1499,10 +1634,14 @@
           <t>PRM_HI_DHS_PERL</t>
         </is>
       </c>
-      <c r="B100" s="2" t="n"/>
-      <c r="C100" s="7" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>be6ec70b8a7f46f7d6a06b554ecf50a16d437e6fcc62de6201fc88ef77c8e589</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>8305796017bbaf420b6513131705df553987508840f6d6d3a9c273856bce6a88</t>
         </is>
       </c>
     </row>
@@ -1521,10 +1660,14 @@
           <t>PRM_ID_DHW_MPEL</t>
         </is>
       </c>
-      <c r="B102" s="2" t="n"/>
-      <c r="C102" s="7" t="inlineStr">
+      <c r="B102" s="2" t="inlineStr">
         <is>
           <t>8305796017bbaf420b6513131705df553987508840f6d6d3a9c273856bce6a88</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
     </row>
@@ -1534,8 +1677,12 @@
           <t>PRM_IL_DHFS_PSL</t>
         </is>
       </c>
-      <c r="B103" s="2" t="n"/>
-      <c r="C103" s="7" t="inlineStr">
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>d518580384830d59c4970219d50dba21d7f0b9f198158f96e429430b3da34738</t>
+        </is>
+      </c>
+      <c r="C103" s="9" t="inlineStr">
         <is>
           <t>d518580384830d59c4970219d50dba21d7f0b9f198158f96e429430b3da34738</t>
         </is>
@@ -1547,10 +1694,14 @@
           <t>PRM_IN_FSSA_PT</t>
         </is>
       </c>
-      <c r="B104" s="2" t="n"/>
-      <c r="C104" s="7" t="inlineStr">
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>81f0db78033949cad3ca3573547710a1b699b59edb88b8bc054053f87032684e</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
         </is>
       </c>
     </row>
@@ -1560,10 +1711,14 @@
           <t>PRM_KS_DHE_TPL</t>
         </is>
       </c>
-      <c r="B105" s="2" t="n"/>
-      <c r="C105" s="7" t="inlineStr">
+      <c r="B105" s="2" t="inlineStr">
         <is>
           <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>d962c6659ca32c7acfa6e2e62e88e685b1bf650f0abcf62ff6c16f6940865235</t>
         </is>
       </c>
     </row>
@@ -1591,8 +1746,12 @@
           <t>PRM_LA_DOA_DV</t>
         </is>
       </c>
-      <c r="B108" s="2" t="n"/>
-      <c r="C108" s="7" t="inlineStr">
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>f95600dbe4b7515fad7acde4481cc0cce4decf85732e935968f8d2b0f9d293a1</t>
+        </is>
+      </c>
+      <c r="C108" s="9" t="inlineStr">
         <is>
           <t>f95600dbe4b7515fad7acde4481cc0cce4decf85732e935968f8d2b0f9d293a1</t>
         </is>
@@ -1605,7 +1764,11 @@
         </is>
       </c>
       <c r="B109" s="2" t="n"/>
-      <c r="C109" s="3" t="n"/>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -1613,10 +1776,14 @@
           <t>PRM_MD_BPW_CB</t>
         </is>
       </c>
-      <c r="B110" s="2" t="n"/>
-      <c r="C110" s="7" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>66e1bef0bd7b07e2497af494d0c4a293672323135f876763fdf12792132d8a22</t>
         </is>
       </c>
     </row>
@@ -1626,10 +1793,14 @@
           <t>PRM_MD_MDH_MSPL</t>
         </is>
       </c>
-      <c r="B111" s="2" t="n"/>
-      <c r="C111" s="7" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>66e1bef0bd7b07e2497af494d0c4a293672323135f876763fdf12792132d8a22</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>b4471a9a0184a21afb00ed648b5850b0828fc314f5b4cae05a5baf17dd62ce06</t>
         </is>
       </c>
     </row>
@@ -1639,12 +1810,12 @@
           <t>PRM_MI_DHHS_SPL</t>
         </is>
       </c>
-      <c r="B112" s="2" t="n"/>
-      <c r="C112" s="7" t="inlineStr">
+      <c r="B112" s="2" t="inlineStr">
         <is>
           <t>b4471a9a0184a21afb00ed648b5850b0828fc314f5b4cae05a5baf17dd62ce06</t>
         </is>
       </c>
+      <c r="C112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -1661,8 +1832,12 @@
           <t>PRM_MS_DM_SPL</t>
         </is>
       </c>
-      <c r="B114" s="2" t="n"/>
-      <c r="C114" s="7" t="inlineStr">
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>db305a14a585151ef7c215b3f9b378664b2eb4b3e871056308243818a6038dc4</t>
+        </is>
+      </c>
+      <c r="C114" s="9" t="inlineStr">
         <is>
           <t>db305a14a585151ef7c215b3f9b378664b2eb4b3e871056308243818a6038dc4</t>
         </is>
@@ -1674,8 +1849,12 @@
           <t>PRM_MT_DPHHS_TMP</t>
         </is>
       </c>
-      <c r="B115" s="2" t="n"/>
-      <c r="C115" s="7" t="inlineStr">
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>dbeac7ceb2efa6046986b3277977fbedd6a46b087b148a31c3917fa47acc50a3</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
         <is>
           <t>dbeac7ceb2efa6046986b3277977fbedd6a46b087b148a31c3917fa47acc50a3</t>
         </is>
@@ -1687,12 +1866,12 @@
           <t>PRM_NC_DA_DV</t>
         </is>
       </c>
-      <c r="B116" s="2" t="n"/>
-      <c r="C116" s="7" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>6534abc9a6ec370e98171e10302ac7098e92763d88fc2b73859a865ec21b352a</t>
         </is>
       </c>
+      <c r="C116" s="3" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -1700,10 +1879,14 @@
           <t>PRM_NC_DHHS_EPL</t>
         </is>
       </c>
-      <c r="B117" s="2" t="n"/>
-      <c r="C117" s="7" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>f2a539248a18f0e2c14ce9bf1844814b3d299d0437b34c5bc9389552d7cf921b</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>6534abc9a6ec370e98171e10302ac7098e92763d88fc2b73859a865ec21b352a</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1897,11 @@
         </is>
       </c>
       <c r="B118" s="2" t="n"/>
-      <c r="C118" s="3" t="n"/>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>f2a539248a18f0e2c14ce9bf1844814b3d299d0437b34c5bc9389552d7cf921b</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -1731,10 +1918,14 @@
           <t>PRM_NJ_MFD_PER</t>
         </is>
       </c>
-      <c r="B120" s="2" t="n"/>
-      <c r="C120" s="7" t="inlineStr">
+      <c r="B120" s="2" t="inlineStr">
         <is>
           <t>c77698286bc91feca5d67a11f6d92f9e4aa427bf32b5b18bf7c4cb91b5ede995</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>ff757e8d46ef6c3713b4acc711c8702408f3275f666935af2d5db55661733797</t>
         </is>
       </c>
     </row>
@@ -1744,8 +1935,12 @@
           <t>PRM_NV_DHHS_MSL</t>
         </is>
       </c>
-      <c r="B121" s="2" t="n"/>
-      <c r="C121" s="7" t="inlineStr">
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
+        </is>
+      </c>
+      <c r="C121" s="9" t="inlineStr">
         <is>
           <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
         </is>
@@ -1766,8 +1961,12 @@
           <t>PRM_NY_DOL_DL</t>
         </is>
       </c>
-      <c r="B123" s="2" t="n"/>
-      <c r="C123" s="7" t="inlineStr">
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
         <is>
           <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
         </is>
@@ -1788,8 +1987,12 @@
           <t>PRM_OR_BOLI_IC</t>
         </is>
       </c>
-      <c r="B125" s="2" t="n"/>
-      <c r="C125" s="7" t="inlineStr">
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
         <is>
           <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
         </is>
@@ -1802,7 +2005,11 @@
         </is>
       </c>
       <c r="B126" s="2" t="n"/>
-      <c r="C126" s="3" t="n"/>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
+          <t>b1ffb6182e3b39e2edae006e55d56d0abbdc953766c90a3d5e0ca5d3e298e569</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -1819,12 +2026,12 @@
           <t>PRM_SC_SFAA_SD</t>
         </is>
       </c>
-      <c r="B128" s="2" t="n"/>
-      <c r="C128" s="7" t="inlineStr">
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>123eff993c9338db4825258e12a99915dd30c2dfaa85d2bd722eb4aa7fa934a8</t>
         </is>
       </c>
+      <c r="C128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -1850,12 +2057,12 @@
           <t>PRM_TX_TC_DVL</t>
         </is>
       </c>
-      <c r="B131" s="2" t="n"/>
-      <c r="C131" s="7" t="inlineStr">
+      <c r="B131" s="2" t="inlineStr">
         <is>
           <t>c339d5a4c816c8fe640bb33245ee683bbe1a03ddecbd211cd33b5770b2ff3bee</t>
         </is>
       </c>
+      <c r="C131" s="3" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -1863,12 +2070,12 @@
           <t>PRM_WA_DOLI_DC</t>
         </is>
       </c>
-      <c r="B132" s="2" t="n"/>
-      <c r="C132" s="7" t="inlineStr">
+      <c r="B132" s="2" t="inlineStr">
         <is>
           <t>6ad1c795d9459f2cfe15aac0c268ada6ca5eb2af707b379d525f43f76baaeecd</t>
         </is>
       </c>
+      <c r="C132" s="3" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -1876,10 +2083,14 @@
           <t>PRM_WA_HCA_PTEL</t>
         </is>
       </c>
-      <c r="B133" s="2" t="n"/>
-      <c r="C133" s="7" t="inlineStr">
+      <c r="B133" s="2" t="inlineStr">
         <is>
           <t>286743119741e3d8569d95f3a661d97f580208f5dcdfe028c3fb0dc9c73fd511</t>
+        </is>
+      </c>
+      <c r="C133" s="8" t="inlineStr">
+        <is>
+          <t>c339d5a4c816c8fe640bb33245ee683bbe1a03ddecbd211cd33b5770b2ff3bee</t>
         </is>
       </c>
     </row>
@@ -1889,8 +2100,12 @@
           <t>PRM_WI_DOT_DSIC</t>
         </is>
       </c>
-      <c r="B134" s="2" t="n"/>
-      <c r="C134" s="7" t="inlineStr">
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>3dcb502f532343574ae604f9293110487e36dcb657946afe8b6cf4b8d2676ec3</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
         <is>
           <t>3dcb502f532343574ae604f9293110487e36dcb657946afe8b6cf4b8d2676ec3</t>
         </is>
@@ -1902,12 +2117,12 @@
           <t>PRM_WV_DHHR_PSE</t>
         </is>
       </c>
-      <c r="B135" s="2" t="n"/>
-      <c r="C135" s="7" t="inlineStr">
+      <c r="B135" s="2" t="inlineStr">
         <is>
           <t>5e4a8fa56aad55b9202fcc9a27f2cdcc4c633fee759c57cc555eb8c37672d8aa</t>
         </is>
       </c>
+      <c r="C135" s="3" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -1925,7 +2140,11 @@
         </is>
       </c>
       <c r="B137" s="2" t="n"/>
-      <c r="C137" s="3" t="n"/>
+      <c r="C137" s="7" t="inlineStr">
+        <is>
+          <t>93e0500aba96ec8070238428036e3b086ba000b945defae61b5c4bb9f82f6fe2</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -1933,8 +2152,12 @@
           <t>QA_MOI_SANCTIONS_LIST</t>
         </is>
       </c>
-      <c r="B138" s="2" t="n"/>
-      <c r="C138" s="7" t="inlineStr">
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>661b722535b10cdf0de28fa5864d8c1c864c1c6f60b7b6c8e98e793ad73aff4e</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
         <is>
           <t>661b722535b10cdf0de28fa5864d8c1c864c1c6f60b7b6c8e98e793ad73aff4e</t>
         </is>
@@ -1964,8 +2187,12 @@
           <t>SECO_SWISS_MOLDOVA</t>
         </is>
       </c>
-      <c r="B141" s="2" t="n"/>
-      <c r="C141" s="7" t="inlineStr">
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>c32fc899559630a399ab8c58c81bcd18273925656dfeba91aa0b780795c122de</t>
+        </is>
+      </c>
+      <c r="C141" s="9" t="inlineStr">
         <is>
           <t>c32fc899559630a399ab8c58c81bcd18273925656dfeba91aa0b780795c122de</t>
         </is>
@@ -1977,10 +2204,14 @@
           <t>SG_ACRA_SUSPENSION</t>
         </is>
       </c>
-      <c r="B142" s="2" t="n"/>
-      <c r="C142" s="7" t="inlineStr">
+      <c r="B142" s="2" t="inlineStr">
         <is>
           <t>1868912449868cc8572bc8ff350dda7706018bb79c95ed9bd84b486e3ff293eb</t>
+        </is>
+      </c>
+      <c r="C142" s="8" t="inlineStr">
+        <is>
+          <t>25b89a575dc4068f1dfec36d7ba1a3d5fe2494aff373a8a56da95394b68e5665</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2231,11 @@
         </is>
       </c>
       <c r="B144" s="2" t="n"/>
-      <c r="C144" s="3" t="n"/>
+      <c r="C144" s="7" t="inlineStr">
+        <is>
+          <t>1868912449868cc8572bc8ff350dda7706018bb79c95ed9bd84b486e3ff293eb</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -2044,12 +2279,12 @@
           <t>TR_MTF_ARTICLE_7</t>
         </is>
       </c>
-      <c r="B149" s="2" t="n"/>
-      <c r="C149" s="7" t="inlineStr">
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>25b89a575dc4068f1dfec36d7ba1a3d5fe2494aff373a8a56da95394b68e5665</t>
         </is>
       </c>
+      <c r="C149" s="3" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -2057,12 +2292,12 @@
           <t>TREAS_FINCEN_ADVISORY</t>
         </is>
       </c>
-      <c r="B150" s="2" t="n"/>
-      <c r="C150" s="7" t="inlineStr">
+      <c r="B150" s="2" t="inlineStr">
         <is>
           <t>93e0500aba96ec8070238428036e3b086ba000b945defae61b5c4bb9f82f6fe2</t>
         </is>
       </c>
+      <c r="C150" s="3" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -2088,8 +2323,12 @@
           <t>TT_FIU_HAITI</t>
         </is>
       </c>
-      <c r="B153" s="2" t="n"/>
-      <c r="C153" s="7" t="inlineStr">
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
+        </is>
+      </c>
+      <c r="C153" s="9" t="inlineStr">
         <is>
           <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
         </is>
@@ -2101,12 +2340,12 @@
           <t>TW_CBI_MW</t>
         </is>
       </c>
-      <c r="B154" s="2" t="n"/>
-      <c r="C154" s="7" t="inlineStr">
+      <c r="B154" s="2" t="inlineStr">
         <is>
           <t>0c2763e4cbb15e86537a56cc3876313f65777ca39f265ec814950470fb611097</t>
         </is>
       </c>
+      <c r="C154" s="3" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -2114,8 +2353,12 @@
           <t>TW_FSC_EA</t>
         </is>
       </c>
-      <c r="B155" s="2" t="n"/>
-      <c r="C155" s="7" t="inlineStr">
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>b1ceda46805367b39634e4c4c7cc43c3220072f4f0ecaf8d1d32c2541725ad05</t>
+        </is>
+      </c>
+      <c r="C155" s="9" t="inlineStr">
         <is>
           <t>b1ceda46805367b39634e4c4c7cc43c3220072f4f0ecaf8d1d32c2541725ad05</t>
         </is>
@@ -2145,8 +2388,12 @@
           <t>US_CBP_UEL</t>
         </is>
       </c>
-      <c r="B158" s="2" t="n"/>
-      <c r="C158" s="7" t="inlineStr">
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>26da235ced9cc83f9bb8e10c17e32985abea89a92308573ce687e82f3f04a8ee</t>
+        </is>
+      </c>
+      <c r="C158" s="9" t="inlineStr">
         <is>
           <t>26da235ced9cc83f9bb8e10c17e32985abea89a92308573ce687e82f3f04a8ee</t>
         </is>
@@ -2186,7 +2433,11 @@
         </is>
       </c>
       <c r="B162" s="2" t="n"/>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="7" t="inlineStr">
+        <is>
+          <t>2b4810348de492ff6092b30166f4cdb8f6dddabaedaab77645a2c42f91dd59ae</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2195,7 +2446,11 @@
         </is>
       </c>
       <c r="B163" s="2" t="n"/>
-      <c r="C163" s="3" t="n"/>
+      <c r="C163" s="7" t="inlineStr">
+        <is>
+          <t>ec2f8e26229154812be2b7017fa9338ad6d18abb8f0b43c37aad614f29f357ca</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -2239,12 +2494,12 @@
           <t>US_NJL_IDA</t>
         </is>
       </c>
-      <c r="B168" s="2" t="n"/>
-      <c r="C168" s="7" t="inlineStr">
+      <c r="B168" s="2" t="inlineStr">
         <is>
           <t>2748bfdae093fc22c38d7699d0eff0027b36ddf5e474388d9ea5a6e350a445e1</t>
         </is>
       </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2252,8 +2507,12 @@
           <t>US_OGT_SCI</t>
         </is>
       </c>
-      <c r="B169" s="2" t="n"/>
-      <c r="C169" s="7" t="inlineStr">
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
+      <c r="C169" s="9" t="inlineStr">
         <is>
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
@@ -2265,10 +2524,14 @@
           <t>US_PDGS_IFP_LIST</t>
         </is>
       </c>
-      <c r="B170" s="2" t="n"/>
-      <c r="C170" s="7" t="inlineStr">
+      <c r="B170" s="2" t="inlineStr">
         <is>
           <t>00c79ba93df9be776984c966c36f797929bd6a347c893f65a4ef8567333a9741</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>2748bfdae093fc22c38d7699d0eff0027b36ddf5e474388d9ea5a6e350a445e1</t>
         </is>
       </c>
     </row>
@@ -2296,10 +2559,14 @@
           <t>US_SS_MWF</t>
         </is>
       </c>
-      <c r="B173" s="2" t="n"/>
-      <c r="C173" s="7" t="inlineStr">
+      <c r="B173" s="2" t="inlineStr">
         <is>
           <t>20b6f000a58e180c0b81853a00e148d6b13055577deebdf160357c20623f1856</t>
+        </is>
+      </c>
+      <c r="C173" s="8" t="inlineStr">
+        <is>
+          <t>1ba563242d86f569400dc5c8b948ecba34917949c7d7f064a73257fcbb0f61a3</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2576,12 @@
           <t>ZA_FIC_SANCTIONS</t>
         </is>
       </c>
-      <c r="B174" s="2" t="n"/>
-      <c r="C174" s="7" t="inlineStr">
+      <c r="B174" s="2" t="inlineStr">
         <is>
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
+      <c r="C174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -2332,7 +2599,11 @@
         </is>
       </c>
       <c r="B176" s="2" t="n"/>
-      <c r="C176" s="3" t="n"/>
+      <c r="C176" s="7" t="inlineStr">
+        <is>
+          <t>063521cb0e62665252346b33902ad1274d97d37e288297551c6217fa8bedd5ab</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2345,7 +2616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2648,6 +2919,30 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:58:00</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>109</v>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>DOS_SDP, EE_FSA_IA, EE_MFA_BELARUS, EE_MFA_HR, EE_MFA_RUSSIA, ES_BOS_SANCTIONS, EU_ECB_SANCTIONS, GB_OFSI_TR_MP, GE_MOJ_OTKHOZORIA_TATUNASHVILI_LIST, GG_GFSC_DD, HK_ICAC_WL, LV_FIU_SANCTIONED_SUBJECTS, MY_BNM_WANTED, MY_BNM_WARNING_LETTERS, MY_MHA_MOHA_LIST, MY_SCM_WANTED, OIG_MOST_WANTED, OM_NCTC_LL, PA_TREAS_SCI, PRM_AK_DHSS_EPL, PRM_CA_DHCS_SIPL, PRM_GA_DCH_EIE, PRM_HI_DHS_PERL, PRM_ID_DHW_MPEL, PRM_IN_FSSA_PT, PRM_KS_DHE_TPL, PRM_MD_BPW_CB, PRM_MD_MDH_MSPL, PRM_NC_DHHS_EPL, PRM_NJ_MFD_PER, PRM_WA_HCA_PTEL, SG_ACRA_SUSPENSION, US_PDGS_IFP_LIST, US_SS_MWF</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 13:34 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -692,10 +692,10 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>a59d5c4f20b63854c4df3bed0310fbc2bee93af59c0a18d5e3a954e4d601fa20</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
+          <t>e89f3f0ef4c85b90f58f5699acd19a0b412df4204c446142abe65d3e72d8792e</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>e89f3f0ef4c85b90f58f5699acd19a0b412df4204c446142abe65d3e72d8792e</t>
         </is>
@@ -735,12 +735,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
+          <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
           <t>b49d363fea1698d0cbff18399767485ef9270ddbee1a1a7670e125462d0fab47</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
         </is>
       </c>
     </row>
@@ -752,12 +752,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
+          <t>0c241186f021344adbd702a2597e4d322f38402077d02d4cb067154deca3c935</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>0c241186f021344adbd702a2597e4d322f38402077d02d4cb067154deca3c935</t>
+          <t>e4fd0143e2c774595c60b307396849dcd3b6d001cc3dbdc82ba7c3557f9aa3e0</t>
         </is>
       </c>
     </row>
@@ -769,12 +769,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>3648e39ea4020a4c625e5ab32c984527fa3a57fae67d0f069ca00c73e8cf2108</t>
+          <t>d8f3558dd1ac550c39aa10e9be6893687468f705c175768e30209db3c85a4c53</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>d8f3558dd1ac550c39aa10e9be6893687468f705c175768e30209db3c85a4c53</t>
+          <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
         </is>
       </c>
     </row>
@@ -786,12 +786,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>af0ba49273abf20fc9ad6a958c30545abe715f6dc086c82b8f42f8ffc293693a</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
           <t>d8f3558dd1ac550c39aa10e9be6893687468f705c175768e30209db3c85a4c53</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>af0ba49273abf20fc9ad6a958c30545abe715f6dc086c82b8f42f8ffc293693a</t>
         </is>
       </c>
     </row>
@@ -812,12 +812,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>0c241186f021344adbd702a2597e4d322f38402077d02d4cb067154deca3c935</t>
+          <t>b49d363fea1698d0cbff18399767485ef9270ddbee1a1a7670e125462d0fab47</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>b49d363fea1698d0cbff18399767485ef9270ddbee1a1a7670e125462d0fab47</t>
+          <t>c0c6681a21424a4a5ca75742f21cf8b600e126382235be07570849cca7280559</t>
         </is>
       </c>
     </row>
@@ -847,12 +847,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>5d37089637de415d106d75fe99fe62d723ed7b89ef99a428890c802ab1c191b5</t>
+          <t>e4fd0143e2c774595c60b307396849dcd3b6d001cc3dbdc82ba7c3557f9aa3e0</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>e4fd0143e2c774595c60b307396849dcd3b6d001cc3dbdc82ba7c3557f9aa3e0</t>
+          <t>fc1c7d780c98b18ff17a0109a346316342ad815013763d1bd245c37b08b5c02b</t>
         </is>
       </c>
     </row>
@@ -867,9 +867,9 @@
           <t>fc1c7d780c98b18ff17a0109a346316342ad815013763d1bd245c37b08b5c02b</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>fc1c7d780c98b18ff17a0109a346316342ad815013763d1bd245c37b08b5c02b</t>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>0c241186f021344adbd702a2597e4d322f38402077d02d4cb067154deca3c935</t>
         </is>
       </c>
     </row>
@@ -935,12 +935,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>c1adf73082a14d642ad9d2f6151af5efab3d3d6531a018b71f3e5c60dfe8d75f</t>
+          <t>727002db8d4a852527360740f82788109fe7990d5fa865436f209de32dcc55e7</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>727002db8d4a852527360740f82788109fe7990d5fa865436f209de32dcc55e7</t>
+          <t>f68f761f9f6c1ee104f780c7cf09c125c05aa1405a1f7d03a63e2ddf7d5820fc</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>5faecf12b7eb37185942d9c032d2327c8b32c5289aa0f7f0ef6e1b7090294289</t>
+          <t>f68f761f9f6c1ee104f780c7cf09c125c05aa1405a1f7d03a63e2ddf7d5820fc</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>f68f761f9f6c1ee104f780c7cf09c125c05aa1405a1f7d03a63e2ddf7d5820fc</t>
+          <t>9ae7d6ec85e9dc4953355a9e61bd3d799eac5b91115e1e13c8383d17e25046b1</t>
         </is>
       </c>
     </row>
@@ -986,12 +986,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>f68f761f9f6c1ee104f780c7cf09c125c05aa1405a1f7d03a63e2ddf7d5820fc</t>
+          <t>c1adf73082a14d642ad9d2f6151af5efab3d3d6531a018b71f3e5c60dfe8d75f</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>c1adf73082a14d642ad9d2f6151af5efab3d3d6531a018b71f3e5c60dfe8d75f</t>
+          <t>5faecf12b7eb37185942d9c032d2327c8b32c5289aa0f7f0ef6e1b7090294289</t>
         </is>
       </c>
     </row>
@@ -1010,12 +1010,12 @@
           <t>IE_CBI_PN</t>
         </is>
       </c>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>5faecf12b7eb37185942d9c032d2327c8b32c5289aa0f7f0ef6e1b7090294289</t>
         </is>
       </c>
+      <c r="C48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1225,8 +1225,12 @@
           <t>KR_MFA_SAKP</t>
         </is>
       </c>
-      <c r="B71" s="2" t="n"/>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>1bcc6af80e092cfff3bab5b083f086f509af69dad954ab936d4313969dcd4e40</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
         <is>
           <t>1bcc6af80e092cfff3bab5b083f086f509af69dad954ab936d4313969dcd4e40</t>
         </is>
@@ -1262,12 +1266,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>7dae12401bb47769506966ad734f2330840383de6cb3853bd22cb145afcbe42c</t>
+          <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
+          <t>3ae9521463edeb0eced6c79ff99009318a605b4c1875f0764719306e04b1d6b6</t>
         </is>
       </c>
     </row>
@@ -1323,12 +1327,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
+          <t>501f8dae7648ae91a810b9e2387294b2e8fe418312f99ff9b4f0f6caa7ffb7f2</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
           <t>fca0e583b4034a443821bda0f8672738cac6e91c078cc019c1969be960766078</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
-          <t>501f8dae7648ae91a810b9e2387294b2e8fe418312f99ff9b4f0f6caa7ffb7f2</t>
         </is>
       </c>
     </row>
@@ -1340,10 +1344,10 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
-        </is>
-      </c>
-      <c r="C80" s="8" t="inlineStr">
+          <t>d8f34f8159cd03ad5427029f244e099e16fc9360c9ac8ffa2c5dbead3b47159e</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
         <is>
           <t>d8f34f8159cd03ad5427029f244e099e16fc9360c9ac8ffa2c5dbead3b47159e</t>
         </is>
@@ -1360,9 +1364,9 @@
           <t>78f4d0658968d9676c029dba90d3b95426f1e07ccf85a59586fabaad7c90e167</t>
         </is>
       </c>
-      <c r="C81" s="9" t="inlineStr">
-        <is>
-          <t>78f4d0658968d9676c029dba90d3b95426f1e07ccf85a59586fabaad7c90e167</t>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1395,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>35c866a9bb3c47bb5d4f9332453c133e924f3932f83220aadeb413629f43ac62</t>
+          <t>f2018bda949c182b01fea214a8fa8e5b690d9b815ab1edf972be3f4a38b8748c</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>f2018bda949c182b01fea214a8fa8e5b690d9b815ab1edf972be3f4a38b8748c</t>
+          <t>b21e47b98b75d4565361957498a1199d8b206bb154e60696995c30930a561fbb</t>
         </is>
       </c>
     </row>
@@ -1442,9 +1446,9 @@
           <t>2d4327f484c5c1f2080dca40f9492c3fa6bfa0bb542764f35d2a84f55e1c27cd</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>2d4327f484c5c1f2080dca40f9492c3fa6bfa0bb542764f35d2a84f55e1c27cd</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
     </row>
@@ -1456,12 +1460,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>791423cc63028135230f287fa0af735437fd8ee36797c8f46e64e1cddd98e0ae</t>
+          <t>3495c2faad0dc9d8a6f151c33ce11f7e60b1666b812ac20d8075e55e8e2ae20c</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>3495c2faad0dc9d8a6f151c33ce11f7e60b1666b812ac20d8075e55e8e2ae20c</t>
+          <t>2d4327f484c5c1f2080dca40f9492c3fa6bfa0bb542764f35d2a84f55e1c27cd</t>
         </is>
       </c>
     </row>
@@ -1476,11 +1480,7 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C89" s="9" t="inlineStr">
-        <is>
-          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
-        </is>
-      </c>
+      <c r="C89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -1490,12 +1490,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
+          <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
+          <t>3495c2faad0dc9d8a6f151c33ce11f7e60b1666b812ac20d8075e55e8e2ae20c</t>
         </is>
       </c>
     </row>
@@ -1505,12 +1505,12 @@
           <t>PL_MOF_SRM</t>
         </is>
       </c>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="7" t="inlineStr">
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>51b08ef9938bb45ef673804ba89c5e5eea02391599e8736362ae7626dff1ed94</t>
         </is>
       </c>
+      <c r="C91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -1520,12 +1520,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
+          <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
           <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,11 @@
           <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1571,9 +1575,9 @@
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
         </is>
       </c>
     </row>
@@ -1588,11 +1592,7 @@
           <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>51b08ef9938bb45ef673804ba89c5e5eea02391599e8736362ae7626dff1ed94</t>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+          <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
         </is>
       </c>
     </row>
@@ -1628,12 +1628,12 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>be6ec70b8a7f46f7d6a06b554ecf50a16d437e6fcc62de6201fc88ef77c8e589</t>
+          <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
+          <t>51b08ef9938bb45ef673804ba89c5e5eea02391599e8736362ae7626dff1ed94</t>
         </is>
       </c>
     </row>
@@ -1657,9 +1657,9 @@
           <t>8305796017bbaf420b6513131705df553987508840f6d6d3a9c273856bce6a88</t>
         </is>
       </c>
-      <c r="C102" s="9" t="inlineStr">
-        <is>
-          <t>8305796017bbaf420b6513131705df553987508840f6d6d3a9c273856bce6a88</t>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>81f0db78033949cad3ca3573547710a1b699b59edb88b8bc054053f87032684e</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1671,12 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>d518580384830d59c4970219d50dba21d7f0b9f198158f96e429430b3da34738</t>
+          <t>81f0db78033949cad3ca3573547710a1b699b59edb88b8bc054053f87032684e</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>81f0db78033949cad3ca3573547710a1b699b59edb88b8bc054053f87032684e</t>
+          <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
         </is>
       </c>
     </row>
@@ -1688,12 +1688,12 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>81f0db78033949cad3ca3573547710a1b699b59edb88b8bc054053f87032684e</t>
+          <t>d518580384830d59c4970219d50dba21d7f0b9f198158f96e429430b3da34738</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>d518580384830d59c4970219d50dba21d7f0b9f198158f96e429430b3da34738</t>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
     </row>
@@ -1705,12 +1705,12 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
+          <t>be6ec70b8a7f46f7d6a06b554ecf50a16d437e6fcc62de6201fc88ef77c8e589</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>be6ec70b8a7f46f7d6a06b554ecf50a16d437e6fcc62de6201fc88ef77c8e589</t>
+          <t>d962c6659ca32c7acfa6e2e62e88e685b1bf650f0abcf62ff6c16f6940865235</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,11 @@
         </is>
       </c>
       <c r="B107" s="2" t="n"/>
-      <c r="C107" s="3" t="n"/>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -1740,12 +1744,12 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
+          <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
           <t>f95600dbe4b7515fad7acde4481cc0cce4decf85732e935968f8d2b0f9d293a1</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
         </is>
       </c>
     </row>
@@ -1766,12 +1770,12 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
+          <t>f95600dbe4b7515fad7acde4481cc0cce4decf85732e935968f8d2b0f9d293a1</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>f95600dbe4b7515fad7acde4481cc0cce4decf85732e935968f8d2b0f9d293a1</t>
+          <t>66e1bef0bd7b07e2497af494d0c4a293672323135f876763fdf12792132d8a22</t>
         </is>
       </c>
     </row>
@@ -1786,9 +1790,9 @@
           <t>66e1bef0bd7b07e2497af494d0c4a293672323135f876763fdf12792132d8a22</t>
         </is>
       </c>
-      <c r="C111" s="9" t="inlineStr">
-        <is>
-          <t>66e1bef0bd7b07e2497af494d0c4a293672323135f876763fdf12792132d8a22</t>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>b4471a9a0184a21afb00ed648b5850b0828fc314f5b4cae05a5baf17dd62ce06</t>
         </is>
       </c>
     </row>
@@ -1800,10 +1804,10 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>b4471a9a0184a21afb00ed648b5850b0828fc314f5b4cae05a5baf17dd62ce06</t>
-        </is>
-      </c>
-      <c r="C112" s="8" t="inlineStr">
+          <t>091c5f744a480cbffc96747165b46d16a0180df4c0522e8af991c41236244665</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="inlineStr">
         <is>
           <t>091c5f744a480cbffc96747165b46d16a0180df4c0522e8af991c41236244665</t>
         </is>
@@ -1829,9 +1833,9 @@
           <t>db305a14a585151ef7c215b3f9b378664b2eb4b3e871056308243818a6038dc4</t>
         </is>
       </c>
-      <c r="C114" s="9" t="inlineStr">
-        <is>
-          <t>db305a14a585151ef7c215b3f9b378664b2eb4b3e871056308243818a6038dc4</t>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>dbeac7ceb2efa6046986b3277977fbedd6a46b087b148a31c3917fa47acc50a3</t>
         </is>
       </c>
     </row>
@@ -1846,11 +1850,7 @@
           <t>dbeac7ceb2efa6046986b3277977fbedd6a46b087b148a31c3917fa47acc50a3</t>
         </is>
       </c>
-      <c r="C115" s="9" t="inlineStr">
-        <is>
-          <t>dbeac7ceb2efa6046986b3277977fbedd6a46b087b148a31c3917fa47acc50a3</t>
-        </is>
-      </c>
+      <c r="C115" s="3" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
+          <t>f2a539248a18f0e2c14ce9bf1844814b3d299d0437b34c5bc9389552d7cf921b</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
           <t>6534abc9a6ec370e98171e10302ac7098e92763d88fc2b73859a865ec21b352a</t>
-        </is>
-      </c>
-      <c r="C116" s="8" t="inlineStr">
-        <is>
-          <t>f2a539248a18f0e2c14ce9bf1844814b3d299d0437b34c5bc9389552d7cf921b</t>
         </is>
       </c>
     </row>
@@ -1877,12 +1877,12 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
+          <t>6534abc9a6ec370e98171e10302ac7098e92763d88fc2b73859a865ec21b352a</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
           <t>f2a539248a18f0e2c14ce9bf1844814b3d299d0437b34c5bc9389552d7cf921b</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t>6534abc9a6ec370e98171e10302ac7098e92763d88fc2b73859a865ec21b352a</t>
         </is>
       </c>
     </row>
@@ -1892,10 +1892,14 @@
           <t>PRM_ND_DHS_MPEL</t>
         </is>
       </c>
-      <c r="B118" s="2" t="n"/>
-      <c r="C118" s="7" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr">
         <is>
           <t>ff757e8d46ef6c3713b4acc711c8702408f3275f666935af2d5db55661733797</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>e5deec3b2a708f576bc8dde34283ccac1a0cd8a401b26689ff7b015d365ff182</t>
         </is>
       </c>
     </row>
@@ -1905,12 +1909,12 @@
           <t>PRM_NH_DHHS_MPESL</t>
         </is>
       </c>
-      <c r="B119" s="2" t="n"/>
-      <c r="C119" s="7" t="inlineStr">
+      <c r="B119" s="2" t="inlineStr">
         <is>
           <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
         </is>
       </c>
+      <c r="C119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -1923,9 +1927,9 @@
           <t>c77698286bc91feca5d67a11f6d92f9e4aa427bf32b5b18bf7c4cb91b5ede995</t>
         </is>
       </c>
-      <c r="C120" s="9" t="inlineStr">
-        <is>
-          <t>c77698286bc91feca5d67a11f6d92f9e4aa427bf32b5b18bf7c4cb91b5ede995</t>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
         </is>
       </c>
     </row>
@@ -1937,12 +1941,12 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
+          <t>e5deec3b2a708f576bc8dde34283ccac1a0cd8a401b26689ff7b015d365ff182</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t>e5deec3b2a708f576bc8dde34283ccac1a0cd8a401b26689ff7b015d365ff182</t>
+          <t>ff757e8d46ef6c3713b4acc711c8702408f3275f666935af2d5db55661733797</t>
         </is>
       </c>
     </row>
@@ -1963,10 +1967,10 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="inlineStr">
+          <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
         <is>
           <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
         </is>
@@ -1992,7 +1996,11 @@
           <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
         </is>
       </c>
-      <c r="C125" s="3" t="n"/>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -2000,8 +2008,12 @@
           <t>PRM_PA_DGS_DSL</t>
         </is>
       </c>
-      <c r="B126" s="2" t="n"/>
-      <c r="C126" s="7" t="inlineStr">
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>b1ffb6182e3b39e2edae006e55d56d0abbdc953766c90a3d5e0ca5d3e298e569</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
         <is>
           <t>b1ffb6182e3b39e2edae006e55d56d0abbdc953766c90a3d5e0ca5d3e298e569</t>
         </is>
@@ -2013,12 +2025,12 @@
           <t>PRM_SC_DHHS_EPL</t>
         </is>
       </c>
-      <c r="B127" s="2" t="n"/>
-      <c r="C127" s="7" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
         <is>
           <t>93e0500aba96ec8070238428036e3b086ba000b945defae61b5c4bb9f82f6fe2</t>
         </is>
       </c>
+      <c r="C127" s="3" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -2028,12 +2040,12 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>123eff993c9338db4825258e12a99915dd30c2dfaa85d2bd722eb4aa7fa934a8</t>
+          <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
+          <t>93e0500aba96ec8070238428036e3b086ba000b945defae61b5c4bb9f82f6fe2</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2056,11 @@
         </is>
       </c>
       <c r="B129" s="2" t="n"/>
-      <c r="C129" s="3" t="n"/>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t>123eff993c9338db4825258e12a99915dd30c2dfaa85d2bd722eb4aa7fa934a8</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -2063,14 +2079,10 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>c339d5a4c816c8fe640bb33245ee683bbe1a03ddecbd211cd33b5770b2ff3bee</t>
-        </is>
-      </c>
-      <c r="C131" s="8" t="inlineStr">
-        <is>
           <t>123eff993c9338db4825258e12a99915dd30c2dfaa85d2bd722eb4aa7fa934a8</t>
         </is>
       </c>
+      <c r="C131" s="3" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -2080,14 +2092,10 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>6ad1c795d9459f2cfe15aac0c268ada6ca5eb2af707b379d525f43f76baaeecd</t>
-        </is>
-      </c>
-      <c r="C132" s="8" t="inlineStr">
-        <is>
           <t>c339d5a4c816c8fe640bb33245ee683bbe1a03ddecbd211cd33b5770b2ff3bee</t>
         </is>
       </c>
+      <c r="C132" s="3" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -2097,12 +2105,12 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>286743119741e3d8569d95f3a661d97f580208f5dcdfe028c3fb0dc9c73fd511</t>
+          <t>25b89a575dc4068f1dfec36d7ba1a3d5fe2494aff373a8a56da95394b68e5665</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t>25b89a575dc4068f1dfec36d7ba1a3d5fe2494aff373a8a56da95394b68e5665</t>
+          <t>c339d5a4c816c8fe640bb33245ee683bbe1a03ddecbd211cd33b5770b2ff3bee</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2125,11 @@
           <t>3dcb502f532343574ae604f9293110487e36dcb657946afe8b6cf4b8d2676ec3</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>6ad1c795d9459f2cfe15aac0c268ada6ca5eb2af707b379d525f43f76baaeecd</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2182,12 +2194,12 @@
           <t>SECO_SWISS_HAMAS</t>
         </is>
       </c>
-      <c r="B140" s="2" t="n"/>
-      <c r="C140" s="7" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>c32fc899559630a399ab8c58c81bcd18273925656dfeba91aa0b780795c122de</t>
         </is>
       </c>
+      <c r="C140" s="3" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -2197,14 +2209,10 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>c32fc899559630a399ab8c58c81bcd18273925656dfeba91aa0b780795c122de</t>
-        </is>
-      </c>
-      <c r="C141" s="8" t="inlineStr">
-        <is>
           <t>5e4a8fa56aad55b9202fcc9a27f2cdcc4c633fee759c57cc555eb8c37672d8aa</t>
         </is>
       </c>
+      <c r="C141" s="3" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -2235,7 +2243,11 @@
         </is>
       </c>
       <c r="B144" s="2" t="n"/>
-      <c r="C144" s="3" t="n"/>
+      <c r="C144" s="7" t="inlineStr">
+        <is>
+          <t>e419e93b2a8c35ef2ac2651ae84039dca8ef527fbac2b31aeb290cf855114018</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -2244,7 +2256,11 @@
         </is>
       </c>
       <c r="B145" s="2" t="n"/>
-      <c r="C145" s="3" t="n"/>
+      <c r="C145" s="7" t="inlineStr">
+        <is>
+          <t>c32fc899559630a399ab8c58c81bcd18273925656dfeba91aa0b780795c122de</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -2284,7 +2300,11 @@
           <t>25b89a575dc4068f1dfec36d7ba1a3d5fe2494aff373a8a56da95394b68e5665</t>
         </is>
       </c>
-      <c r="C149" s="3" t="n"/>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>1868912449868cc8572bc8ff350dda7706018bb79c95ed9bd84b486e3ff293eb</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -2297,7 +2317,11 @@
           <t>93e0500aba96ec8070238428036e3b086ba000b945defae61b5c4bb9f82f6fe2</t>
         </is>
       </c>
-      <c r="C150" s="3" t="n"/>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>59dc968b9f1615ef168dd2329aea04b20fddfdd3da0a6446e3672cc305c43782</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -2306,7 +2330,11 @@
         </is>
       </c>
       <c r="B151" s="2" t="n"/>
-      <c r="C151" s="3" t="n"/>
+      <c r="C151" s="7" t="inlineStr">
+        <is>
+          <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -2314,10 +2342,14 @@
           <t>TT_FIU_DPRK</t>
         </is>
       </c>
-      <c r="B152" s="2" t="n"/>
-      <c r="C152" s="7" t="inlineStr">
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>59dc968b9f1615ef168dd2329aea04b20fddfdd3da0a6446e3672cc305c43782</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>b1ceda46805367b39634e4c4c7cc43c3220072f4f0ecaf8d1d32c2541725ad05</t>
         </is>
       </c>
     </row>
@@ -2329,14 +2361,10 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
-        </is>
-      </c>
-      <c r="C153" s="8" t="inlineStr">
-        <is>
           <t>b1ceda46805367b39634e4c4c7cc43c3220072f4f0ecaf8d1d32c2541725ad05</t>
         </is>
       </c>
+      <c r="C153" s="3" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -2346,12 +2374,12 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>0c2763e4cbb15e86537a56cc3876313f65777ca39f265ec814950470fb611097</t>
+          <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
         </is>
       </c>
       <c r="C154" s="8" t="inlineStr">
         <is>
-          <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
+          <t>da6d77469efe81d9044efb805152571642352f4aa39698f2bd517753db6e4545</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2394,11 @@
           <t>b1ceda46805367b39634e4c4c7cc43c3220072f4f0ecaf8d1d32c2541725ad05</t>
         </is>
       </c>
-      <c r="C155" s="3" t="n"/>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>7b2894d384353c6cf8eaa05bbe1b60004f3585c496c0d365a395e6900afe6cb0</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -2394,10 +2426,10 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>26da235ced9cc83f9bb8e10c17e32985abea89a92308573ce687e82f3f04a8ee</t>
-        </is>
-      </c>
-      <c r="C158" s="8" t="inlineStr">
+          <t>2b4810348de492ff6092b30166f4cdb8f6dddabaedaab77645a2c42f91dd59ae</t>
+        </is>
+      </c>
+      <c r="C158" s="9" t="inlineStr">
         <is>
           <t>2b4810348de492ff6092b30166f4cdb8f6dddabaedaab77645a2c42f91dd59ae</t>
         </is>
@@ -2436,10 +2468,14 @@
           <t>US_DOT_MOST_WANTED</t>
         </is>
       </c>
-      <c r="B162" s="2" t="n"/>
-      <c r="C162" s="7" t="inlineStr">
+      <c r="B162" s="2" t="inlineStr">
         <is>
           <t>26da235ced9cc83f9bb8e10c17e32985abea89a92308573ce687e82f3f04a8ee</t>
+        </is>
+      </c>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2532,12 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>2748bfdae093fc22c38d7699d0eff0027b36ddf5e474388d9ea5a6e350a445e1</t>
+          <t>625833d34b5c5ae7af74e338048290ddeb9f0641df34c24c02d513631a92affd</t>
         </is>
       </c>
       <c r="C168" s="8" t="inlineStr">
         <is>
-          <t>625833d34b5c5ae7af74e338048290ddeb9f0641df34c24c02d513631a92affd</t>
+          <t>d1c8a1a9e4a2bc96cb33befae759d29a5356e0b4cd3acfd42df6df75e70e70e3</t>
         </is>
       </c>
     </row>
@@ -2513,12 +2549,12 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+          <t>063521cb0e62665252346b33902ad1274d97d37e288297551c6217fa8bedd5ab</t>
         </is>
       </c>
       <c r="C169" s="8" t="inlineStr">
         <is>
-          <t>063521cb0e62665252346b33902ad1274d97d37e288297551c6217fa8bedd5ab</t>
+          <t>625833d34b5c5ae7af74e338048290ddeb9f0641df34c24c02d513631a92affd</t>
         </is>
       </c>
     </row>
@@ -2530,12 +2566,12 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>00c79ba93df9be776984c966c36f797929bd6a347c893f65a4ef8567333a9741</t>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
       <c r="C170" s="8" t="inlineStr">
         <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+          <t>063521cb0e62665252346b33902ad1274d97d37e288297551c6217fa8bedd5ab</t>
         </is>
       </c>
     </row>
@@ -2565,12 +2601,12 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>20b6f000a58e180c0b81853a00e148d6b13055577deebdf160357c20623f1856</t>
+          <t>2748bfdae093fc22c38d7699d0eff0027b36ddf5e474388d9ea5a6e350a445e1</t>
         </is>
       </c>
       <c r="C173" s="8" t="inlineStr">
         <is>
-          <t>2748bfdae093fc22c38d7699d0eff0027b36ddf5e474388d9ea5a6e350a445e1</t>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
     </row>
@@ -2582,12 +2618,12 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+          <t>1ba563242d86f569400dc5c8b948ecba34917949c7d7f064a73257fcbb0f61a3</t>
         </is>
       </c>
       <c r="C174" s="8" t="inlineStr">
         <is>
-          <t>1ba563242d86f569400dc5c8b948ecba34917949c7d7f064a73257fcbb0f61a3</t>
+          <t>20b6f000a58e180c0b81853a00e148d6b13055577deebdf160357c20623f1856</t>
         </is>
       </c>
     </row>
@@ -2606,12 +2642,12 @@
           <t>ZA_FSCA_EA</t>
         </is>
       </c>
-      <c r="B176" s="2" t="n"/>
-      <c r="C176" s="7" t="inlineStr">
+      <c r="B176" s="2" t="inlineStr">
         <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
+      <c r="C176" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2624,7 +2660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2951,6 +2987,30 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01 13:21:01</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>EE_MFA_BELARUS, EE_MFA_HR, EE_MFA_RUSSIA, ES_BOS_SANCTIONS, ES_WA_CNMV, EU_ECB_SANCTIONS, EU_EIB_LOE, GB_OFSI_TR_MP, GE_MOJ_OTKHOZORIA_TATUNASHVILI_LIST, HK_ICAC_WL, MC_BT_NAFL, MY_MHA_MOHA_LIST, MY_SCM_WANTED, NG_NIGSAC_ENTITIES, OIG_MOST_WANTED, OM_NCTC_LL, PE_MEF_DISQUALIFIED_SUPPLIERS, PRM_AK_DHSS_EPL, PRM_CA_DIR_DC, PRM_GA_DCH_EIE, PRM_HI_DHS_PERL, PRM_ID_DHW_MPEL, PRM_IL_DHFS_PSL, PRM_IN_FSSA_PT, PRM_KS_DHE_TPL, PRM_LA_DOA_DV, PRM_MD_BPW_CB, PRM_MD_MDH_MSPL, PRM_MS_DM_SPL, PRM_NC_DA_DV, PRM_NC_DHHS_EPL, PRM_ND_DHS_MPEL, PRM_NJ_MFD_PER, PRM_NV_DHHS_MSL, PRM_OR_BOLI_IC, PRM_SC_SFAA_SD, PRM_WA_HCA_PTEL, PRM_WI_DOT_DSIC, TR_MTF_ARTICLE_7, TREAS_FINCEN_ADVISORY, TT_FIU_DPRK, TW_CBI_MW, TW_FSC_EA, US_DOT_MOST_WANTED, US_NJL_IDA, US_OGT_SCI, US_PDGS_IFP_LIST, US_SS_MWF, ZA_FIC_SANCTIONS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 13:48 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -695,11 +695,7 @@
           <t>e89f3f0ef4c85b90f58f5699acd19a0b412df4204c446142abe65d3e72d8792e</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>e89f3f0ef4c85b90f58f5699acd19a0b412df4204c446142abe65d3e72d8792e</t>
-        </is>
-      </c>
+      <c r="C24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -721,11 +717,7 @@
           <t>8f5304ae2f1524f86cd781e21057001c1e3be04eda31d4469e88d0453e93c4b9</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>8f5304ae2f1524f86cd781e21057001c1e3be04eda31d4469e88d0453e93c4b9</t>
-        </is>
-      </c>
+      <c r="C26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -735,14 +727,10 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
           <t>b49d363fea1698d0cbff18399767485ef9270ddbee1a1a7670e125462d0fab47</t>
         </is>
       </c>
+      <c r="C27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -752,14 +740,10 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>0c241186f021344adbd702a2597e4d322f38402077d02d4cb067154deca3c935</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
           <t>e4fd0143e2c774595c60b307396849dcd3b6d001cc3dbdc82ba7c3557f9aa3e0</t>
         </is>
       </c>
+      <c r="C28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -769,14 +753,10 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>d8f3558dd1ac550c39aa10e9be6893687468f705c175768e30209db3c85a4c53</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
           <t>218699a04a01aab623a77dade4c954dfdf5f161c226000f1f66f12104d70ddfb</t>
         </is>
       </c>
+      <c r="C29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -786,14 +766,10 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>af0ba49273abf20fc9ad6a958c30545abe715f6dc086c82b8f42f8ffc293693a</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
           <t>d8f3558dd1ac550c39aa10e9be6893687468f705c175768e30209db3c85a4c53</t>
         </is>
       </c>
+      <c r="C30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -812,14 +788,10 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>b49d363fea1698d0cbff18399767485ef9270ddbee1a1a7670e125462d0fab47</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
           <t>c0c6681a21424a4a5ca75742f21cf8b600e126382235be07570849cca7280559</t>
         </is>
       </c>
+      <c r="C32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -847,14 +819,10 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>e4fd0143e2c774595c60b307396849dcd3b6d001cc3dbdc82ba7c3557f9aa3e0</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
           <t>fc1c7d780c98b18ff17a0109a346316342ad815013763d1bd245c37b08b5c02b</t>
         </is>
       </c>
+      <c r="C35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -864,14 +832,10 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>fc1c7d780c98b18ff17a0109a346316342ad815013763d1bd245c37b08b5c02b</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
           <t>0c241186f021344adbd702a2597e4d322f38402077d02d4cb067154deca3c935</t>
         </is>
       </c>
+      <c r="C36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -935,14 +899,10 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>727002db8d4a852527360740f82788109fe7990d5fa865436f209de32dcc55e7</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
           <t>f68f761f9f6c1ee104f780c7cf09c125c05aa1405a1f7d03a63e2ddf7d5820fc</t>
         </is>
       </c>
+      <c r="C43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -952,14 +912,10 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>f68f761f9f6c1ee104f780c7cf09c125c05aa1405a1f7d03a63e2ddf7d5820fc</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
           <t>9ae7d6ec85e9dc4953355a9e61bd3d799eac5b91115e1e13c8383d17e25046b1</t>
         </is>
       </c>
+      <c r="C44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -972,11 +928,7 @@
           <t>a14038d31708de4f8a5594ee7ca8166907baa31b2cd2e63811bb6fefb7b4c0a0</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>a14038d31708de4f8a5594ee7ca8166907baa31b2cd2e63811bb6fefb7b4c0a0</t>
-        </is>
-      </c>
+      <c r="C45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -986,14 +938,10 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>c1adf73082a14d642ad9d2f6151af5efab3d3d6531a018b71f3e5c60dfe8d75f</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
           <t>5faecf12b7eb37185942d9c032d2327c8b32c5289aa0f7f0ef6e1b7090294289</t>
         </is>
       </c>
+      <c r="C46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1230,11 +1178,7 @@
           <t>1bcc6af80e092cfff3bab5b083f086f509af69dad954ab936d4313969dcd4e40</t>
         </is>
       </c>
-      <c r="C71" s="9" t="inlineStr">
-        <is>
-          <t>1bcc6af80e092cfff3bab5b083f086f509af69dad954ab936d4313969dcd4e40</t>
-        </is>
-      </c>
+      <c r="C71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -1266,14 +1210,10 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
           <t>3ae9521463edeb0eced6c79ff99009318a605b4c1875f0764719306e04b1d6b6</t>
         </is>
       </c>
+      <c r="C74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -1327,14 +1267,10 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>501f8dae7648ae91a810b9e2387294b2e8fe418312f99ff9b4f0f6caa7ffb7f2</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
           <t>fca0e583b4034a443821bda0f8672738cac6e91c078cc019c1969be960766078</t>
         </is>
       </c>
+      <c r="C79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -1347,11 +1283,7 @@
           <t>d8f34f8159cd03ad5427029f244e099e16fc9360c9ac8ffa2c5dbead3b47159e</t>
         </is>
       </c>
-      <c r="C80" s="9" t="inlineStr">
-        <is>
-          <t>d8f34f8159cd03ad5427029f244e099e16fc9360c9ac8ffa2c5dbead3b47159e</t>
-        </is>
-      </c>
+      <c r="C80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -1361,14 +1293,10 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>78f4d0658968d9676c029dba90d3b95426f1e07ccf85a59586fabaad7c90e167</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="inlineStr">
-        <is>
           <t>704036ff26f0814f40d217e04008850bf67888dd39d5b2a064bfabc0288ea17f</t>
         </is>
       </c>
+      <c r="C81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -1381,11 +1309,7 @@
           <t>97abe1aac9218570b13169c1395f3ecd2651f8d2efa03e9b0c91b0da8f307afb</t>
         </is>
       </c>
-      <c r="C82" s="9" t="inlineStr">
-        <is>
-          <t>97abe1aac9218570b13169c1395f3ecd2651f8d2efa03e9b0c91b0da8f307afb</t>
-        </is>
-      </c>
+      <c r="C82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -1395,14 +1319,10 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>f2018bda949c182b01fea214a8fa8e5b690d9b815ab1edf972be3f4a38b8748c</t>
-        </is>
-      </c>
-      <c r="C83" s="8" t="inlineStr">
-        <is>
           <t>b21e47b98b75d4565361957498a1199d8b206bb154e60696995c30930a561fbb</t>
         </is>
       </c>
+      <c r="C83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -1443,10 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2d4327f484c5c1f2080dca40f9492c3fa6bfa0bb542764f35d2a84f55e1c27cd</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
+          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
@@ -1460,14 +1380,10 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>3495c2faad0dc9d8a6f151c33ce11f7e60b1666b812ac20d8075e55e8e2ae20c</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="inlineStr">
-        <is>
           <t>2d4327f484c5c1f2080dca40f9492c3fa6bfa0bb542764f35d2a84f55e1c27cd</t>
         </is>
       </c>
+      <c r="C88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -1490,14 +1406,10 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="inlineStr">
-        <is>
           <t>3495c2faad0dc9d8a6f151c33ce11f7e60b1666b812ac20d8075e55e8e2ae20c</t>
         </is>
       </c>
+      <c r="C90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -1520,12 +1432,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
+          <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
+          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
     </row>
@@ -1558,9 +1470,9 @@
           <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
         </is>
       </c>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
         </is>
       </c>
     </row>
@@ -1572,14 +1484,10 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
           <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
         </is>
       </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1592,7 +1500,11 @@
           <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1611,14 +1523,10 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C99" s="8" t="inlineStr">
-        <is>
           <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
         </is>
       </c>
+      <c r="C99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -1628,14 +1536,10 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
-        </is>
-      </c>
-      <c r="C100" s="8" t="inlineStr">
-        <is>
           <t>51b08ef9938bb45ef673804ba89c5e5eea02391599e8736362ae7626dff1ed94</t>
         </is>
       </c>
+      <c r="C100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -1654,14 +1558,10 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>8305796017bbaf420b6513131705df553987508840f6d6d3a9c273856bce6a88</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
           <t>81f0db78033949cad3ca3573547710a1b699b59edb88b8bc054053f87032684e</t>
         </is>
       </c>
+      <c r="C102" s="3" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -1671,14 +1571,10 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>81f0db78033949cad3ca3573547710a1b699b59edb88b8bc054053f87032684e</t>
-        </is>
-      </c>
-      <c r="C103" s="8" t="inlineStr">
-        <is>
           <t>6424d492b6c78b72695a4ecdcca3175b8db0a1516d284c2b1daba763c60a9d49</t>
         </is>
       </c>
+      <c r="C103" s="3" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -1688,14 +1584,10 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>d518580384830d59c4970219d50dba21d7f0b9f198158f96e429430b3da34738</t>
-        </is>
-      </c>
-      <c r="C104" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C104" s="3" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -1705,14 +1597,10 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>be6ec70b8a7f46f7d6a06b554ecf50a16d437e6fcc62de6201fc88ef77c8e589</t>
-        </is>
-      </c>
-      <c r="C105" s="8" t="inlineStr">
-        <is>
           <t>d962c6659ca32c7acfa6e2e62e88e685b1bf650f0abcf62ff6c16f6940865235</t>
         </is>
       </c>
+      <c r="C105" s="3" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -1729,12 +1617,12 @@
           <t>PRM_LA_DH_AAL</t>
         </is>
       </c>
-      <c r="B107" s="2" t="n"/>
-      <c r="C107" s="7" t="inlineStr">
+      <c r="B107" s="2" t="inlineStr">
         <is>
           <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
         </is>
       </c>
+      <c r="C107" s="3" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -1744,14 +1632,10 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>96d2ce493afbd69c573a79cb0f93dd0691a390de292afbbb55980ef9c912dfdd</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
           <t>f95600dbe4b7515fad7acde4481cc0cce4decf85732e935968f8d2b0f9d293a1</t>
         </is>
       </c>
+      <c r="C108" s="3" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -1770,14 +1654,10 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>f95600dbe4b7515fad7acde4481cc0cce4decf85732e935968f8d2b0f9d293a1</t>
-        </is>
-      </c>
-      <c r="C110" s="8" t="inlineStr">
-        <is>
           <t>66e1bef0bd7b07e2497af494d0c4a293672323135f876763fdf12792132d8a22</t>
         </is>
       </c>
+      <c r="C110" s="3" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -1787,14 +1667,10 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>66e1bef0bd7b07e2497af494d0c4a293672323135f876763fdf12792132d8a22</t>
-        </is>
-      </c>
-      <c r="C111" s="8" t="inlineStr">
-        <is>
           <t>b4471a9a0184a21afb00ed648b5850b0828fc314f5b4cae05a5baf17dd62ce06</t>
         </is>
       </c>
+      <c r="C111" s="3" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -1807,11 +1683,7 @@
           <t>091c5f744a480cbffc96747165b46d16a0180df4c0522e8af991c41236244665</t>
         </is>
       </c>
-      <c r="C112" s="9" t="inlineStr">
-        <is>
-          <t>091c5f744a480cbffc96747165b46d16a0180df4c0522e8af991c41236244665</t>
-        </is>
-      </c>
+      <c r="C112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -1830,14 +1702,10 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>db305a14a585151ef7c215b3f9b378664b2eb4b3e871056308243818a6038dc4</t>
-        </is>
-      </c>
-      <c r="C114" s="8" t="inlineStr">
-        <is>
           <t>dbeac7ceb2efa6046986b3277977fbedd6a46b087b148a31c3917fa47acc50a3</t>
         </is>
       </c>
+      <c r="C114" s="3" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -1860,14 +1728,10 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>f2a539248a18f0e2c14ce9bf1844814b3d299d0437b34c5bc9389552d7cf921b</t>
-        </is>
-      </c>
-      <c r="C116" s="8" t="inlineStr">
-        <is>
           <t>6534abc9a6ec370e98171e10302ac7098e92763d88fc2b73859a865ec21b352a</t>
         </is>
       </c>
+      <c r="C116" s="3" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -1877,14 +1741,10 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>6534abc9a6ec370e98171e10302ac7098e92763d88fc2b73859a865ec21b352a</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
           <t>f2a539248a18f0e2c14ce9bf1844814b3d299d0437b34c5bc9389552d7cf921b</t>
         </is>
       </c>
+      <c r="C117" s="3" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -1894,14 +1754,10 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>ff757e8d46ef6c3713b4acc711c8702408f3275f666935af2d5db55661733797</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
           <t>e5deec3b2a708f576bc8dde34283ccac1a0cd8a401b26689ff7b015d365ff182</t>
         </is>
       </c>
+      <c r="C118" s="3" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -1924,14 +1780,10 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>c77698286bc91feca5d67a11f6d92f9e4aa427bf32b5b18bf7c4cb91b5ede995</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
           <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
         </is>
       </c>
+      <c r="C120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -1941,14 +1793,10 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>e5deec3b2a708f576bc8dde34283ccac1a0cd8a401b26689ff7b015d365ff182</t>
-        </is>
-      </c>
-      <c r="C121" s="8" t="inlineStr">
-        <is>
           <t>ff757e8d46ef6c3713b4acc711c8702408f3275f666935af2d5db55661733797</t>
         </is>
       </c>
+      <c r="C121" s="3" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -1970,11 +1818,7 @@
           <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
         </is>
       </c>
-      <c r="C123" s="9" t="inlineStr">
-        <is>
-          <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
-        </is>
-      </c>
+      <c r="C123" s="3" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -1993,14 +1837,10 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>5c8cbcffef0ccd2817c80bb9756ae5433aaa9c1a221d5f5db2a9f4c8a76b0074</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="inlineStr">
-        <is>
           <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
         </is>
       </c>
+      <c r="C125" s="3" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -2013,11 +1853,7 @@
           <t>b1ffb6182e3b39e2edae006e55d56d0abbdc953766c90a3d5e0ca5d3e298e569</t>
         </is>
       </c>
-      <c r="C126" s="9" t="inlineStr">
-        <is>
-          <t>b1ffb6182e3b39e2edae006e55d56d0abbdc953766c90a3d5e0ca5d3e298e569</t>
-        </is>
-      </c>
+      <c r="C126" s="3" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -2040,14 +1876,10 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>6e156cb46055efeb7285838436937b4d8b35d5a4df422d02a1f15e9f411dfd07</t>
-        </is>
-      </c>
-      <c r="C128" s="8" t="inlineStr">
-        <is>
           <t>93e0500aba96ec8070238428036e3b086ba000b945defae61b5c4bb9f82f6fe2</t>
         </is>
       </c>
+      <c r="C128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -2055,12 +1887,12 @@
           <t>PRM_TN_OPI_TPL</t>
         </is>
       </c>
-      <c r="B129" s="2" t="n"/>
-      <c r="C129" s="7" t="inlineStr">
+      <c r="B129" s="2" t="inlineStr">
         <is>
           <t>123eff993c9338db4825258e12a99915dd30c2dfaa85d2bd722eb4aa7fa934a8</t>
         </is>
       </c>
+      <c r="C129" s="3" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -2105,14 +1937,10 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>25b89a575dc4068f1dfec36d7ba1a3d5fe2494aff373a8a56da95394b68e5665</t>
-        </is>
-      </c>
-      <c r="C133" s="8" t="inlineStr">
-        <is>
           <t>c339d5a4c816c8fe640bb33245ee683bbe1a03ddecbd211cd33b5770b2ff3bee</t>
         </is>
       </c>
+      <c r="C133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -2122,14 +1950,10 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>3dcb502f532343574ae604f9293110487e36dcb657946afe8b6cf4b8d2676ec3</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
           <t>6ad1c795d9459f2cfe15aac0c268ada6ca5eb2af707b379d525f43f76baaeecd</t>
         </is>
       </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2173,11 +1997,7 @@
           <t>661b722535b10cdf0de28fa5864d8c1c864c1c6f60b7b6c8e98e793ad73aff4e</t>
         </is>
       </c>
-      <c r="C138" s="9" t="inlineStr">
-        <is>
-          <t>661b722535b10cdf0de28fa5864d8c1c864c1c6f60b7b6c8e98e793ad73aff4e</t>
-        </is>
-      </c>
+      <c r="C138" s="3" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -2242,12 +2062,12 @@
           <t>SG_SGX_WATCH_LIST</t>
         </is>
       </c>
-      <c r="B144" s="2" t="n"/>
-      <c r="C144" s="7" t="inlineStr">
+      <c r="B144" s="2" t="inlineStr">
         <is>
           <t>e419e93b2a8c35ef2ac2651ae84039dca8ef527fbac2b31aeb290cf855114018</t>
         </is>
       </c>
+      <c r="C144" s="3" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -2255,12 +2075,12 @@
           <t>TH_AMLO_SANCTIONS</t>
         </is>
       </c>
-      <c r="B145" s="2" t="n"/>
-      <c r="C145" s="7" t="inlineStr">
+      <c r="B145" s="2" t="inlineStr">
         <is>
           <t>c32fc899559630a399ab8c58c81bcd18273925656dfeba91aa0b780795c122de</t>
         </is>
       </c>
+      <c r="C145" s="3" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -2297,14 +2117,10 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>25b89a575dc4068f1dfec36d7ba1a3d5fe2494aff373a8a56da95394b68e5665</t>
-        </is>
-      </c>
-      <c r="C149" s="8" t="inlineStr">
-        <is>
           <t>1868912449868cc8572bc8ff350dda7706018bb79c95ed9bd84b486e3ff293eb</t>
         </is>
       </c>
+      <c r="C149" s="3" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -2314,14 +2130,10 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>93e0500aba96ec8070238428036e3b086ba000b945defae61b5c4bb9f82f6fe2</t>
-        </is>
-      </c>
-      <c r="C150" s="8" t="inlineStr">
-        <is>
           <t>59dc968b9f1615ef168dd2329aea04b20fddfdd3da0a6446e3672cc305c43782</t>
         </is>
       </c>
+      <c r="C150" s="3" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -2329,12 +2141,12 @@
           <t>TREAS_FINCEN_PMLC</t>
         </is>
       </c>
-      <c r="B151" s="2" t="n"/>
-      <c r="C151" s="7" t="inlineStr">
+      <c r="B151" s="2" t="inlineStr">
         <is>
           <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
         </is>
       </c>
+      <c r="C151" s="3" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -2344,14 +2156,10 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>59dc968b9f1615ef168dd2329aea04b20fddfdd3da0a6446e3672cc305c43782</t>
-        </is>
-      </c>
-      <c r="C152" s="8" t="inlineStr">
-        <is>
           <t>b1ceda46805367b39634e4c4c7cc43c3220072f4f0ecaf8d1d32c2541725ad05</t>
         </is>
       </c>
+      <c r="C152" s="3" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -2374,14 +2182,10 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>7e72be5eebbf0dd65b2188eb92c19cbb6e8156d46ad26daf0d04477c5765a9cd</t>
-        </is>
-      </c>
-      <c r="C154" s="8" t="inlineStr">
-        <is>
           <t>da6d77469efe81d9044efb805152571642352f4aa39698f2bd517753db6e4545</t>
         </is>
       </c>
+      <c r="C154" s="3" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -2391,14 +2195,10 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>b1ceda46805367b39634e4c4c7cc43c3220072f4f0ecaf8d1d32c2541725ad05</t>
-        </is>
-      </c>
-      <c r="C155" s="8" t="inlineStr">
-        <is>
           <t>7b2894d384353c6cf8eaa05bbe1b60004f3585c496c0d365a395e6900afe6cb0</t>
         </is>
       </c>
+      <c r="C155" s="3" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -2429,11 +2229,7 @@
           <t>2b4810348de492ff6092b30166f4cdb8f6dddabaedaab77645a2c42f91dd59ae</t>
         </is>
       </c>
-      <c r="C158" s="9" t="inlineStr">
-        <is>
-          <t>2b4810348de492ff6092b30166f4cdb8f6dddabaedaab77645a2c42f91dd59ae</t>
-        </is>
-      </c>
+      <c r="C158" s="3" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -2470,10 +2266,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>26da235ced9cc83f9bb8e10c17e32985abea89a92308573ce687e82f3f04a8ee</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
         <is>
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
@@ -2532,14 +2328,10 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>625833d34b5c5ae7af74e338048290ddeb9f0641df34c24c02d513631a92affd</t>
-        </is>
-      </c>
-      <c r="C168" s="8" t="inlineStr">
-        <is>
           <t>d1c8a1a9e4a2bc96cb33befae759d29a5356e0b4cd3acfd42df6df75e70e70e3</t>
         </is>
       </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2549,14 +2341,10 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>063521cb0e62665252346b33902ad1274d97d37e288297551c6217fa8bedd5ab</t>
-        </is>
-      </c>
-      <c r="C169" s="8" t="inlineStr">
-        <is>
           <t>625833d34b5c5ae7af74e338048290ddeb9f0641df34c24c02d513631a92affd</t>
         </is>
       </c>
+      <c r="C169" s="3" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -2566,14 +2354,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
           <t>063521cb0e62665252346b33902ad1274d97d37e288297551c6217fa8bedd5ab</t>
         </is>
       </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2601,14 +2385,10 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>2748bfdae093fc22c38d7699d0eff0027b36ddf5e474388d9ea5a6e350a445e1</t>
-        </is>
-      </c>
-      <c r="C173" s="8" t="inlineStr">
-        <is>
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
+      <c r="C173" s="3" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -2618,14 +2398,10 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>1ba563242d86f569400dc5c8b948ecba34917949c7d7f064a73257fcbb0f61a3</t>
-        </is>
-      </c>
-      <c r="C174" s="8" t="inlineStr">
-        <is>
           <t>20b6f000a58e180c0b81853a00e148d6b13055577deebdf160357c20623f1856</t>
         </is>
       </c>
+      <c r="C174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -2660,7 +2436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3011,6 +2787,30 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-01 13:46:31</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL, PRM_CA_DHCS_SIPL, PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 13:50 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1435,11 +1435,7 @@
           <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
         </is>
       </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1470,11 +1466,7 @@
           <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
         </is>
       </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
-          <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
-        </is>
-      </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1500,11 +1492,7 @@
           <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
         </is>
       </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2331,7 +2319,11 @@
           <t>d1c8a1a9e4a2bc96cb33befae759d29a5356e0b4cd3acfd42df6df75e70e70e3</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="8" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2790,24 +2782,24 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01 13:46:31</t>
+          <t>2026-06-01 13:48:52</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
         <v>175</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>PRM_AK_DHSS_EPL, PRM_CA_DHCS_SIPL, PRM_DC_DDS_PSL</t>
+          <t>US_NJL_IDA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 14:03 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2257,11 +2253,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2316,14 +2308,10 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>d1c8a1a9e4a2bc96cb33befae759d29a5356e0b4cd3acfd42df6df75e70e70e3</t>
-        </is>
-      </c>
-      <c r="C168" s="8" t="inlineStr">
-        <is>
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2428,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2803,6 +2791,30 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:03:16</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 14:08 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1492,7 +1492,11 @@
           <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2257,7 +2261,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2819,6 +2827,30 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:07:17</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 14:16 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1489,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>9d10ee25021a42bf5d64c5056257d78fde267e634a075aaa4b40d812bee48edf</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2323,7 +2319,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2851,6 +2851,30 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:15:19</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 14:41 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1435,7 +1435,11 @@
           <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2257,11 +2261,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2319,11 +2319,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2428,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2875,6 +2871,30 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:39:39</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-01 14:57 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1432,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>a59b2a097818956c8ba4066f31000f8f97da2c138f3d45430248f8ba09d43af8</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1496,7 +1492,11 @@
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2895,6 +2895,30 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:56:17</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-02 06:41 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1489,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2345,7 +2341,11 @@
           <t>063521cb0e62665252346b33902ad1274d97d37e288297551c6217fa8bedd5ab</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2919,6 +2919,30 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-02 06:39:08</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-03 06:51 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1479,7 +1479,11 @@
           <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1492,7 +1496,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2338,14 +2346,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>063521cb0e62665252346b33902ad1274d97d37e288297551c6217fa8bedd5ab</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2943,6 +2947,30 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03 06:50:05</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>PRM_CA_DIR_DC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-04 06:41 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1476,14 +1476,10 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>d24bcb920c479fef7e9345323276b8c74e494c8c47c4cb79a6d6209d6790d05d</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1496,11 +1492,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2265,7 +2257,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2323,7 +2319,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2971,6 +2971,30 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-04 06:40:14</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-05 06:20 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2257,11 +2257,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2319,11 +2315,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2995,6 +2987,30 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-05 06:19:19</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-06 05:53 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1492,7 +1492,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3011,6 +3015,30 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-06 05:52:08</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-07 06:22 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1489,10 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
+          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
         <is>
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
@@ -2319,7 +2319,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3039,6 +3043,30 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07 06:20:57</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-08 06:41 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1492,9 +1492,9 @@
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
     </row>
@@ -2319,11 +2319,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2349,7 +2345,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3067,6 +3067,30 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-08 06:40:03</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL, PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-09 06:08 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1489,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1945,7 +1941,11 @@
           <t>6ad1c795d9459f2cfe15aac0c268ada6ca5eb2af707b379d525f43f76baaeecd</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>abc09d4bcf6148d4e7521e4444b54bddb07efa78af2869619973abaafbd8727d</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2345,11 +2345,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2428,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3091,6 +3087,30 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09 06:06:34</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>PRM_WI_DOT_DSIC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-10 06:22 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1938,14 +1934,10 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>6ad1c795d9459f2cfe15aac0c268ada6ca5eb2af707b379d525f43f76baaeecd</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
           <t>abc09d4bcf6148d4e7521e4444b54bddb07efa78af2869619973abaafbd8727d</t>
         </is>
       </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3111,6 +3103,30 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-10 06:20:50</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-11 06:47 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,7 +1435,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2416,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3127,6 +3135,30 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-11 06:46:00</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-12 06:48 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,9 +1366,9 @@
           <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>ce5320cea37943ae9c38cede17c1bb8490a644937947b34c93961b6a4a552de3</t>
         </is>
       </c>
     </row>
@@ -1435,11 +1435,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2319,7 +2315,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2345,7 +2345,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3159,6 +3163,30 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-12 06:38:14</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-13 06:24 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2ea7462f7ccb5b1cc7bf6c3a8eac5c5c44d4909b2e9404333e9ca330011cf2fe</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>ce5320cea37943ae9c38cede17c1bb8490a644937947b34c93961b6a4a552de3</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2315,11 +2311,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2342,10 +2334,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
+      <c r="C170" s="9" t="inlineStr">
         <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3187,6 +3179,30 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13 06:13:56</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-14 06:46 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>ce5320cea37943ae9c38cede17c1bb8490a644937947b34c93961b6a4a552de3</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>ce5320cea37943ae9c38cede17c1bb8490a644937947b34c93961b6a4a552de3</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1475,7 +1479,11 @@
           <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1488,7 +1496,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2311,7 +2323,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2420,7 +2436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3203,6 +3219,30 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-14 06:36:13</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>PRM_CA_DIR_DC, PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-15 07:15 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1476,14 +1476,10 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>b4c1f7dca66d325bb6b1ceefcac9963e43fdd153dbf20e7318fe1eced1e67127</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1493,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2265,7 +2257,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2323,11 +2319,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2353,11 +2345,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2436,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3243,6 +3231,30 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15 07:14:31</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-16 07:25 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2254,12 +2254,12 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3255,6 +3255,30 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-16 07:23:26</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-17 07:07 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>ce5320cea37943ae9c38cede17c1bb8490a644937947b34c93961b6a4a552de3</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>ce5320cea37943ae9c38cede17c1bb8490a644937947b34c93961b6a4a552de3</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1479,7 +1475,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1492,7 +1492,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2254,14 +2258,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2345,7 +2345,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3279,6 +3283,30 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17 07:05:57</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-18 06:50 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1462,7 +1462,11 @@
           <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1475,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1492,11 +1492,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2261,7 +2257,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2345,11 +2345,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2428,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3307,6 +3303,30 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-18 06:49:07</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>PRM_CA_DHCS_SIPL, US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-19 07:13 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1459,14 +1459,10 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>1865579aaf348bc2a9ad587813f7591b73c2c942a86615170b3554670aad14b4</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
           <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
         </is>
       </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1492,7 +1488,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2254,14 +2254,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2319,7 +2315,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3327,6 +3327,30 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19 07:03:18</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-20 06:27 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>ce5320cea37943ae9c38cede17c1bb8490a644937947b34c93961b6a4a552de3</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>c57a44b518a0468151fd4044f1992aee3f5be525ed3b03904defef6a24ce4bbf</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1485,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2315,11 +2315,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3351,6 +3347,30 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-20 06:17:36</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-21 06:58 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,10 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>ce5320cea37943ae9c38cede17c1bb8490a644937947b34c93961b6a4a552de3</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
+          <t>c57a44b518a0468151fd4044f1992aee3f5be525ed3b03904defef6a24ce4bbf</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>c57a44b518a0468151fd4044f1992aee3f5be525ed3b03904defef6a24ce4bbf</t>
         </is>
@@ -2257,7 +2257,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3371,6 +3375,30 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-21 06:48:22</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-22 07:31 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2254,14 +2254,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2345,7 +2341,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3399,6 +3399,30 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22 07:20:51</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-23 06:14 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>c57a44b518a0468151fd4044f1992aee3f5be525ed3b03904defef6a24ce4bbf</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>c57a44b518a0468151fd4044f1992aee3f5be525ed3b03904defef6a24ce4bbf</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2257,7 +2253,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2338,12 +2338,12 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3423,6 +3423,30 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-23 06:04:04</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-24 06:05 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>c57a44b518a0468151fd4044f1992aee3f5be525ed3b03904defef6a24ce4bbf</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1462,7 +1466,11 @@
           <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1488,7 +1496,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2253,11 +2265,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2338,14 +2346,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3447,6 +3451,30 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24 06:03:53</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-25 06:05 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,10 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>c57a44b518a0468151fd4044f1992aee3f5be525ed3b03904defef6a24ce4bbf</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
+          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
@@ -1466,11 +1466,7 @@
           <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
         </is>
       </c>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
-        </is>
-      </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1496,11 +1492,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3475,6 +3467,30 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25 06:03:38</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-26 06:17 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1466,7 +1466,11 @@
           <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3491,6 +3495,30 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26 06:07:35</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-27 06:01 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1466,11 +1462,7 @@
           <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
         </is>
       </c>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
-        </is>
-      </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2261,7 +2253,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3519,6 +3515,30 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-27 05:51:09</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-28 06:15 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1475,7 +1475,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2250,14 +2254,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3539,6 +3539,30 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28 06:14:21</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-29 06:44 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1475,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2257,7 +2257,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3563,6 +3567,30 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29 06:42:50</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-06-30 06:10 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2257,11 +2253,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2319,7 +2311,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2345,7 +2341,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3591,6 +3591,30 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30 06:07:55</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-01 06:24 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2311,11 +2315,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2341,11 +2341,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3615,6 +3611,30 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01 06:23:03</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-02 06:06 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2315,7 +2315,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2341,7 +2345,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2420,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3635,6 +3643,30 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02 05:56:00</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-03 06:00 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2315,11 +2311,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2345,11 +2337,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2428,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3667,6 +3655,30 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 05:50:25</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-04 05:52 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2416,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3679,6 +3683,30 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-04 05:42:42</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-05 06:11 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3707,6 +3707,30 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-05 06:01:07</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-06 06:35 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1435,7 +1435,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2257,7 +2261,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2315,7 +2323,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2420,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3731,6 +3743,30 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06 06:24:51</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-07 06:14 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1435,11 +1435,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1496,7 +1492,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2258,10 +2258,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
         <is>
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
@@ -2432,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3767,6 +3767,30 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-07 06:04:29</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-08 05:21 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1492,11 +1492,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2261,11 +2257,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2323,11 +2315,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2353,7 +2341,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2432,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3791,6 +3783,30 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08 05:18:15</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-09 06:02 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,11 +1435,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2257,7 +2257,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2341,11 +2345,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3807,6 +3807,30 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:01:14</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-10 06:02 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1466,7 +1466,11 @@
           <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2257,11 +2261,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3831,6 +3831,30 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10 06:00:33</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>PRM_CA_DHCS_SIPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-11 05:12 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1463,14 +1459,10 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>f2e6eafb0dc26ea09580a88acb4e66f1230aff0a9b16bb615ddab33abdb1dce3</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2424,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3855,6 +3847,30 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-11 05:10:36</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-12 05:25 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2253,7 +2253,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2416,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3871,6 +3875,30 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-12 05:24:16</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-13 05:35 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>299b3d805d95dfc5d5a6e678312a8279ff9062e04da666cb140fa7064e613c94</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1488,7 +1492,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2253,11 +2261,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3899,6 +3903,30 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13 05:33:48</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-14 04:58 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,12 +1363,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>e0491af32d9e3135747405fc50a205bdac5777a7a66e325c7386c90694cbb6ca</t>
+          <t>299b3d805d95dfc5d5a6e678312a8279ff9062e04da666cb140fa7064e613c94</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>299b3d805d95dfc5d5a6e678312a8279ff9062e04da666cb140fa7064e613c94</t>
+          <t>f127901255d8922b3e3b73777896976f85b593058bed83038c059164807ea3bf</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1435,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1489,14 +1493,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3927,6 +3927,30 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14 04:48:21</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-15 04:50 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,12 +1363,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>299b3d805d95dfc5d5a6e678312a8279ff9062e04da666cb140fa7064e613c94</t>
+          <t>f127901255d8922b3e3b73777896976f85b593058bed83038c059164807ea3bf</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>f127901255d8922b3e3b73777896976f85b593058bed83038c059164807ea3bf</t>
+          <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
         </is>
       </c>
     </row>
@@ -1435,9 +1435,9 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2261,7 +2265,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2424,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3951,6 +3959,30 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-15 04:48:54</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C64" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-16 04:58 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>f127901255d8922b3e3b73777896976f85b593058bed83038c059164807ea3bf</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1432,12 +1428,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
     </row>
@@ -1496,9 +1492,9 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
         </is>
       </c>
     </row>
@@ -2265,11 +2261,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2432,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3983,6 +3975,30 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16 04:57:19</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL, PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-17 05:21 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,10 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
         <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
@@ -1489,14 +1493,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2345,7 +2345,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3999,6 +4003,30 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 05:11:03</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C66" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-18 04:56 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,9 +1366,9 @@
           <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
         </is>
       </c>
     </row>
@@ -1435,11 +1435,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2342,14 +2338,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4027,6 +4019,30 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-18 04:46:10</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-19 05:20 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,10 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
+          <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
         </is>
@@ -2257,7 +2257,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4043,6 +4047,30 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-19 05:18:53</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C68" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-20 05:48 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1466,7 +1466,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2319,7 +2323,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2424,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4071,6 +4079,30 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20 05:38:10</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-21 05:19 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2261,11 +2261,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2323,11 +2319,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2353,7 +2345,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2432,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4103,6 +4099,30 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-21 05:17:40</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C70" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E70" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-22 05:18 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,9 +1366,9 @@
           <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>6fe257399efe7b321b240a8b8843b1231bc86985c25e9c1213f48abaf5039f45</t>
         </is>
       </c>
     </row>
@@ -1466,11 +1466,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2342,14 +2338,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4123,6 +4115,30 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-22 05:16:33</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-23 05:23 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>6fe257399efe7b321b240a8b8843b1231bc86985c25e9c1213f48abaf5039f45</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1492,7 +1488,11 @@
           <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1941,7 +1941,11 @@
           <t>abc09d4bcf6148d4e7521e4444b54bddb07efa78af2869619973abaafbd8727d</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4139,6 +4143,30 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23 05:21:52</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C72" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL, PRM_WI_DOT_DSIC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-24 05:19 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>6fe257399efe7b321b240a8b8843b1231bc86985c25e9c1213f48abaf5039f45</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>10011a70c0f24a99b32de12cadf343534a18c7f987f60fa2c0f63bf4e013ffeb</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1485,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>c06d19f5eda00e52afe9250b8c414dc96a93234c5472c088b3281cba3d872ca7</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1938,14 +1938,10 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>abc09d4bcf6148d4e7521e4444b54bddb07efa78af2869619973abaafbd8727d</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2261,7 +2257,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2345,7 +2345,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4167,6 +4171,30 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24 05:17:52</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-25 05:22 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>6fe257399efe7b321b240a8b8843b1231bc86985c25e9c1213f48abaf5039f45</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>10011a70c0f24a99b32de12cadf343534a18c7f987f60fa2c0f63bf4e013ffeb</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2257,11 +2257,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2342,14 +2338,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4195,6 +4187,30 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-25 05:11:45</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C74" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-26 05:38 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>10011a70c0f24a99b32de12cadf343534a18c7f987f60fa2c0f63bf4e013ffeb</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>0a8cc025453807f8445db14632cc2b1601ad8598568ccadaa75a3e7b947f938f</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4211,6 +4211,30 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-26 05:28:41</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-27 05:47 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>10011a70c0f24a99b32de12cadf343534a18c7f987f60fa2c0f63bf4e013ffeb</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1492,7 +1488,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4235,6 +4235,30 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-27 05:45:31</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C76" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-28 05:21 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1431,7 +1431,11 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1488,11 +1492,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2257,7 +2257,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2315,7 +2319,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2420,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4259,6 +4267,30 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-28 05:11:28</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C77" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-29 05:20 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1771,7 +1771,11 @@
           <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
         </is>
       </c>
-      <c r="C120" s="3" t="n"/>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>e419e93b2a8c35ef2ac2651ae84039dca8ef527fbac2b31aeb290cf855114018</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -2257,11 +2261,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2319,11 +2319,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2428,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4291,6 +4287,30 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-29 05:18:47</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C78" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>PRM_NJ_MFD_PER</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-30 04:57 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,11 +1435,7 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1768,14 +1768,10 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>781a7266eacf602892461efb2507f70350e765571785afe5f8f0ed43f93f0c81</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
           <t>e419e93b2a8c35ef2ac2651ae84039dca8ef527fbac2b31aeb290cf855114018</t>
         </is>
       </c>
+      <c r="C120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4311,6 +4307,30 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30 04:55:31</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C79" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-07-31 05:42 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1479,7 +1479,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>4786e66777ed63b77ed4abc9849bb29057a71b5a8f0f8751fa2a837c6957c45f</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1492,7 +1496,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2257,7 +2265,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4331,6 +4343,30 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-31 05:32:39</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C80" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D80" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E80" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>PRM_CA_DIR_DC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-01 05:34 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1476,14 +1476,10 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
           <t>4786e66777ed63b77ed4abc9849bb29057a71b5a8f0f8751fa2a837c6957c45f</t>
         </is>
       </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1496,11 +1492,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2265,11 +2257,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2432,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4367,6 +4355,30 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01 05:24:06</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C81" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-02 05:33 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1492,7 +1492,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4379,6 +4383,30 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-02 05:23:33</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C82" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-03 05:48 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1489,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4407,6 +4403,30 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-03 05:38:05</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C83" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-04 05:13 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1435,7 +1435,11 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1492,7 +1496,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2420,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4427,6 +4435,30 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-04 05:11:47</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C84" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E84" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-05 05:13 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1432,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2265,7 +2261,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2323,7 +2323,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2428,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4459,6 +4463,30 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-05 05:11:47</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-06 05:15 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1479,7 +1479,11 @@
           <t>4786e66777ed63b77ed4abc9849bb29057a71b5a8f0f8751fa2a837c6957c45f</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1492,9 +1496,9 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>7f15f935224687830ae62e3a52509b72e8f5bb78ccca381a8a44f84755b71689</t>
         </is>
       </c>
     </row>
@@ -2261,11 +2265,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2323,11 +2323,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2353,7 +2349,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2432,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4487,6 +4487,30 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-06 05:13:42</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C86" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D86" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>PRM_CA_DIR_DC, PRM_DC_DDS_PSL, US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-07 04:24 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1476,14 +1476,10 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>4786e66777ed63b77ed4abc9849bb29057a71b5a8f0f8751fa2a837c6957c45f</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1493,12 +1489,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+          <t>7f15f935224687830ae62e3a52509b72e8f5bb78ccca381a8a44f84755b71689</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>7f15f935224687830ae62e3a52509b72e8f5bb78ccca381a8a44f84755b71689</t>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
     </row>
@@ -2346,14 +2342,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2432,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4511,6 +4503,30 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:23:27</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C87" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-08 03:22 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1489,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>7f15f935224687830ae62e3a52509b72e8f5bb78ccca381a8a44f84755b71689</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4527,6 +4523,30 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-08 03:21:08</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C88" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-09 03:40 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4547,6 +4547,30 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-09 03:29:46</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-10 03:51 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1479,7 +1479,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1492,7 +1496,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2315,7 +2323,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2420,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4571,6 +4583,30 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-10 03:49:54</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C90" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E90" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-11 03:40 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1479,11 +1475,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1493,12 +1485,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
     </row>
@@ -2323,11 +2315,7 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2432,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4607,6 +4595,30 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-11 03:39:15</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-12 04:13 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1475,7 +1479,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1485,14 +1493,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4619,6 +4623,30 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-12 04:03:01</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C92" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E92" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-13 04:08 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4647,6 +4647,30 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-13 04:07:03</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-14 04:04 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,9 +1366,9 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>5b88f7ee490a5df066a024f85de32997bd7c713cb0575b400c35aa6dbecdce9c</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4671,6 +4671,30 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14 04:03:03</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C94" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-15 02:49 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,10 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
+          <t>5b88f7ee490a5df066a024f85de32997bd7c713cb0575b400c35aa6dbecdce9c</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>5b88f7ee490a5df066a024f85de32997bd7c713cb0575b400c35aa6dbecdce9c</t>
         </is>
@@ -1496,7 +1496,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2261,7 +2265,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2424,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4695,6 +4703,30 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-15 02:48:19</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C95" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E95" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-16 02:57 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1479,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1493,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2265,11 +2257,7 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2432,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4727,6 +4715,30 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-16 02:55:50</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C96" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-17 02:57 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>5b88f7ee490a5df066a024f85de32997bd7c713cb0575b400c35aa6dbecdce9c</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>5b88f7ee490a5df066a024f85de32997bd7c713cb0575b400c35aa6dbecdce9c</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1466,7 +1462,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4739,6 +4739,30 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17 02:55:57</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-18 02:53 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>5b88f7ee490a5df066a024f85de32997bd7c713cb0575b400c35aa6dbecdce9c</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>bc0f679a4cfd4cd78dcd4bcd51ca6ff9a474daf5098eaa121b37bbdcb7bfc693</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1462,11 +1466,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1479,7 +1479,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1941,7 +1945,11 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2257,7 +2265,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4763,6 +4775,30 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-18 02:52:07</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C98" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D98" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E98" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-19 02:58 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>5b88f7ee490a5df066a024f85de32997bd7c713cb0575b400c35aa6dbecdce9c</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>bc0f679a4cfd4cd78dcd4bcd51ca6ff9a474daf5098eaa121b37bbdcb7bfc693</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1466,7 +1462,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1945,11 +1945,7 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2262,10 +2258,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
         <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
@@ -2432,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4799,6 +4795,30 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-19 02:57:01</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C99" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D99" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E99" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-20 02:54 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>bc0f679a4cfd4cd78dcd4bcd51ca6ff9a474daf5098eaa121b37bbdcb7bfc693</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>9b6ddb10b3b3e071b29de1567d5df5d8bba42ab4a45d787da543e3c7078cab33</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1462,11 +1466,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1479,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2261,11 +2257,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4819,6 +4811,30 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-20 02:52:34</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C100" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-21 02:59 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,10 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>bc0f679a4cfd4cd78dcd4bcd51ca6ff9a474daf5098eaa121b37bbdcb7bfc693</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
+          <t>9b6ddb10b3b3e071b29de1567d5df5d8bba42ab4a45d787da543e3c7078cab33</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>9b6ddb10b3b3e071b29de1567d5df5d8bba42ab4a45d787da543e3c7078cab33</t>
         </is>
@@ -1435,7 +1435,11 @@
           <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1479,7 +1483,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1941,7 +1949,11 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>e419e93b2a8c35ef2ac2651ae84039dca8ef527fbac2b31aeb290cf855114018</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4835,6 +4847,30 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-21 02:58:20</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C101" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E101" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL, PRM_WI_DOT_DSIC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-22 02:51 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,9 +1366,9 @@
           <t>9b6ddb10b3b3e071b29de1567d5df5d8bba42ab4a45d787da543e3c7078cab33</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>9b6ddb10b3b3e071b29de1567d5df5d8bba42ab4a45d787da543e3c7078cab33</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
         </is>
       </c>
     </row>
@@ -1432,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>7b12de5a66bfa79a190e33c2bb2193c954766bfe0068646cba55e3eabdfe7ca5</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1483,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1946,14 +1938,10 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
           <t>e419e93b2a8c35ef2ac2651ae84039dca8ef527fbac2b31aeb290cf855114018</t>
         </is>
       </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2432,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4871,6 +4859,30 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-22 02:50:10</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C102" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-23 02:59 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>9b6ddb10b3b3e071b29de1567d5df5d8bba42ab4a45d787da543e3c7078cab33</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4883,6 +4883,30 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-23 02:58:10</t>
+        </is>
+      </c>
+      <c r="B103" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C103" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D103" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F103" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-24 03:09 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4907,6 +4907,30 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24 02:59:07</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C104" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-25 03:04 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2420,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4931,6 +4927,30 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-25 02:54:33</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C105" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="F105" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-26 03:01 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1937,7 +1941,11 @@
           <t>e419e93b2a8c35ef2ac2651ae84039dca8ef527fbac2b31aeb290cf855114018</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2416,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4951,6 +4959,30 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-26 03:00:04</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C106" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>PRM_WI_DOT_DSIC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-27 12:27 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,9 +1366,9 @@
           <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
         </is>
       </c>
     </row>
@@ -1938,14 +1938,10 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>e419e93b2a8c35ef2ac2651ae84039dca8ef527fbac2b31aeb290cf855114018</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4983,6 +4979,30 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-27 12:17:23</t>
+        </is>
+      </c>
+      <c r="B107" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C107" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F107" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-28 13:44 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1941,7 +1937,11 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5003,6 +5003,30 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-28 13:42:46</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C108" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-29 08:35 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1431,7 +1431,11 @@
           <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5027,6 +5031,30 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-29 08:34:08</t>
+        </is>
+      </c>
+      <c r="B109" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C109" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-30 07:48 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1428,14 +1428,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>0cb9b0aa66d4a65b19ad0b65c471823789fa9af355996d3b0d8284b9511cbf17</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1479,7 +1475,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5055,6 +5055,30 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-30 07:47:22</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C110" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E110" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-08-31 08:03 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1475,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1941,11 +1941,7 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2261,7 +2257,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5079,6 +5079,30 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-31 08:01:50</t>
+        </is>
+      </c>
+      <c r="B111" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C111" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E111" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-01 07:10 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1466,7 +1462,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>9c5d036ece335c15e680e916cd6cdf2489a92401bc9336ae9837dd292561f567</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1941,7 +1941,11 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F111"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5103,6 +5107,30 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-01 07:09:04</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C112" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E112" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>PRM_CA_DHCS_SIPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-02 06:55 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1459,14 +1463,10 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
           <t>9c5d036ece335c15e680e916cd6cdf2489a92401bc9336ae9837dd292561f567</t>
         </is>
       </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1941,11 +1941,7 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2261,11 +2257,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:F113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5131,6 +5123,30 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-02 06:44:54</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C113" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E113" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-03 06:49 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1941,7 +1941,11 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:F114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5147,6 +5151,30 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-03 06:48:02</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C114" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E114" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-04 07:03 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1492,7 +1492,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1941,11 +1945,7 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5175,6 +5175,30 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-04 06:52:58</t>
+        </is>
+      </c>
+      <c r="B115" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C115" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F115" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-05 06:47 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1428,14 +1428,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1466,7 +1462,11 @@
           <t>9c5d036ece335c15e680e916cd6cdf2489a92401bc9336ae9837dd292561f567</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1492,11 +1492,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5199,6 +5195,30 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 06:37:27</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C116" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>PRM_CA_DHCS_SIPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-06 06:57 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,7 +1435,11 @@
           <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1459,14 +1467,10 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>9c5d036ece335c15e680e916cd6cdf2489a92401bc9336ae9837dd292561f567</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1492,7 +1496,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2257,7 +2265,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5219,6 +5231,30 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-06 06:47:34</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C117" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D117" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E117" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-07 06:57 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>51040edaee08a92064100032b7e982abc3ccad7025779bcab5925ed6ed91765b</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1432,14 +1428,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1496,11 +1488,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1949,7 +1937,11 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2265,11 +2257,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2432,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F117"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5255,6 +5243,30 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07 06:56:21</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C118" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-08 06:53 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F118"/>
+  <dimension ref="A1:F119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5267,6 +5271,30 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-08 06:51:35</t>
+        </is>
+      </c>
+      <c r="B119" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C119" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E119" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-09 07:02 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1435,7 +1435,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2319,7 +2323,11 @@
           <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="8" t="inlineStr">
+        <is>
+          <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2424,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F119"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5295,6 +5303,30 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-09 07:00:42</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C120" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D120" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E120" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL, US_NJL_IDA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-10 06:58 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1432,10 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
         <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
@@ -2320,14 +2320,10 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>2c012cb88b5fc23187222d7e521d22331ce2754cfcd703cfcb15f02b74ee4180</t>
-        </is>
-      </c>
-      <c r="C168" s="8" t="inlineStr">
-        <is>
           <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
         </is>
       </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2432,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5327,6 +5323,30 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-10 06:57:15</t>
+        </is>
+      </c>
+      <c r="B121" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C121" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D121" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E121" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-11 07:07 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1945,11 +1941,7 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F121"/>
+  <dimension ref="A1:F122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5347,6 +5339,30 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 06:57:11</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C122" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D122" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E122" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-12 06:49 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,11 +1435,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1941,7 +1941,11 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5363,6 +5367,30 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-12 06:48:21</t>
+        </is>
+      </c>
+      <c r="B123" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C123" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D123" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E123" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>